<commit_message>
Build salesperson financing discussion agenda
</commit_message>
<xml_diff>
--- a/incoming/Lacks_Store_Data.xlsx
+++ b/incoming/Lacks_Store_Data.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Store Info" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Brands" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Mattresses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Accessories" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SalesNotes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Promotions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Quiz" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Store Info" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brands" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mattresses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accessories" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SalesNotes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6620,7 +6620,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"financing":{"enabled":true,"experience":"payment-choice","offerVersion":"2026-07-30a","verifiedAt":"2026-07-31T16:43:00-05:00","maxAgeDays":7,"sourceUrl":"https://www.lacks.com/financing","applicationUrl":"https://www.lacks.com/credit-application","mexicoInfoUrl":"https://www.lacks.com/faq","mexicoApplicationUrl":{"url":"https://www.lacks.com/mexican-credit-application","verified":false,"note":"Published in Lacks' FAQ but returned 404 on 2026-07-30. Do not render as a link until it resolves; the Mexico card links to mexicoInfoUrl."},"savingsPassPolicy":"specialist_confirm","exactPromotionsEnabled":false,"esReviewStatus":"pending-native-legal-review","allowedSourceHosts":["lacks.com","www.lacks.com","synchrony.com","www.synchrony.com","mysynchrony.com"],"copy":{"eyebrow":{"en":"LACKS PAYMENT CHOICE","es":"OPCIONES DE PAGO LACKS"},"headline":{"en":"Better sleep. More ways to bring it home.","es":"Duerme mejor. Más opciones para llevarlo a casa."},"body":{"en":"Explore promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Options are subject to terms and approval.","es":"Explora financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. Las opciones están sujetas a términos y aprobación."},"cta":{"en":"Explore payment options","es":"Explorar opciones de pago"},"ctaSecondary":{"en":"Review with a Lacks specialist","es":"Revisar con un especialista de Lacks"},"welcomeTagline":{"en":"Flexible ways to bring better sleep home.","es":"Formas flexibles de llevar mejor descanso a casa."},"welcomeSupport":{"en":"Explore payment options after finding your strongest mattress matches.","es":"Explora opciones de pago después de encontrar tus mejores opciones de colchón."},"resultsLead":{"en":"Your strongest mattress match may have more than one way to bring it home.","es":"Tu mejor opción de colchón puede tener más de una forma de llegar a casa."},"resultsAsk":{"en":"Ask my specialist","es":"Preguntar a mi especialista"},"fitFirst":{"en":"Your matches are based on sleep fit — never on payment method.","es":"Tus opciones se basan en tu descanso — nunca en la forma de pago."},"drawerTitle":{"en":"Ways to bring it home","es":"Formas de llevarlo a casa"},"drawerBody":{"en":"This recommendation is based on your sleep fit. When you're ready, Lacks offers more than one way to bring it home.","es":"Esta recomendación se basa en tu descanso. Cuando estés listo, Lacks ofrece más de una forma de llevarlo a casa."},"drawerMark":{"en":"Discuss payment options","es":"Conversar opciones de pago"},"drawerMarked":{"en":"Marked to discuss","es":"Marcado para conversar"},"sleepSystemGuidance":{"en":"Build the sleep setup that fits you first. Your Lacks specialist can then review current payment options for the complete plan.","es":"Primero arma el sistema de sueño que te quede bien. Después, tu especialista de Lacks puede revisar las opciones de pago actuales para el plan completo."},"handoffHeadline":{"en":"Your Sleep Plan. Your Payment Choices.","es":"Tu Plan de Sueño. Tus Opciones de Pago."},"handoffPrivate":{"en":"Continue on your phone — scan to open Lacks' official financing page.","es":"Continúa desde tu teléfono — escanea para abrir la página oficial de financiamiento de Lacks."},"interestPrompt":{"en":"Would you like to review flexible payment options with your Lacks specialist?","es":"¿Te gustaría revisar opciones de pago flexibles con un especialista de Lacks?"},"interestYes":{"en":"Yes, I'm interested","es":"Sí, me interesa"},"interestNotNow":{"en":"Not right now","es":"Ahora no"},"interestMarkedAnnounce":{"en":"Marked for your specialist. Nothing is submitted and no application is started.","es":"Marcado para tu especialista. No se envía nada y no se inicia ninguna solicitud."},"interestNotNowAnnounce":{"en":"Not right now selected. You can change this choice.","es":"Se seleccionó 'Ahora no'. Puedes cambiar esta opción."},"interestClearedAnnounce":{"en":"Selection cleared. Choose again when you're ready.","es":"Se borró la selección. Elige de nuevo cuando quieras."},"staleNotice":{"en":"Current payment options are available from your Lacks specialist.","es":"Tu especialista de Lacks tiene las opciones de pago actuales."},"staleAnnouncement":{"en":"Exact rates and terms are not shown right now. Your Lacks specialist can confirm current payment options in store.","es":"Las tasas y los plazos exactos no se muestran en este momento. Tu especialista de Lacks puede confirmar las opciones de pago actuales en tienda."},"externalNotice":{"en":"Opens lacks.com — a separate site governed by its own terms and privacy policy.","es":"Abre lacks.com — un sitio aparte, regido por sus propios términos y política de privacidad."},"emailHeading":{"en":"Payment options","es":"Opciones de pago"},"emailBody":{"en":"You explored Lacks Payment Choice: promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Final pricing, eligibility, terms, and approval are confirmed by Lacks.","es":"Exploraste las Opciones de Pago Lacks: financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. El precio final, la elegibilidad, los términos y la aprobación los confirma Lacks."},"emailBodyAvailable":{"en":"Lacks Payment Choice offers more than one way to bring it home: promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Final pricing, eligibility, terms, and approval are confirmed by Lacks.","es":"Las Opciones de Pago Lacks ofrecen más de una forma de llevarlo a casa: financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. El precio final, la elegibilidad, los términos y la aprobación los confirma Lacks."},"disclosureFooter":{"en":"All payment options are subject to terms and approval. Advertised purchase minimums, rates, and terms are set by Lacks and its financing partners and may change or end at any time. Your Lacks specialist confirms current details in store.","es":"Todas las opciones de pago están sujetas a términos y aprobación. Los mínimos de compra, tasas y plazos anunciados los establecen Lacks y sus socios financieros y pueden cambiar o terminar en cualquier momento. Tu especialista de Lacks confirma los detalles vigentes en tienda."},"prequalNote":{"en":"See if you prequalify on Lacks' official financing page — prequalification is not approval.","es":"Consulta si precalificas en la página oficial de financiamiento de Lacks — precalificar no es una aprobación."}},"plans":[{"id":"synchrony-9-99-72","kind":"open-end-promotional-credit","provider":"Synchrony","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","apr":9.99,"termMonths":72,"minimumPurchase":500,"channel":"per-current-source","calculationMode":"published-fixed-factor","paymentCalculationEnabled":false,"headline":{"en":"9.99% APR for 72 months","es":"9.99% APR por 72 meses"},"detail":{"en":"On qualifying purchases of $500 or more with the Lacks Furniture Synchrony HOME Credit Card. Fixed monthly payments required. Interest is charged from the purchase date at the reduced APR. The advertised purchase minimum must be met on one receipt; discounts may reduce the purchase below it.","es":"En compras que califiquen de $500 o más con la tarjeta Lacks Furniture Synchrony HOME. Se requieren pagos mensuales fijos. Se cobra interés desde la fecha de compra a la tasa APR reducida. El mínimo de compra anunciado debe cumplirse en un solo recibo; los descuentos pueden reducir la compra por debajo del mínimo."},"disclosure":{"en":"Subject to credit approval. Regular account terms apply to non-promo purchases; for new accounts as of 07/31/2025 the purchase APR is 34.99%, penalty APR 39.99%, minimum interest charge $2. Lacks may alter or discontinue this offer at any time.","es":"Sujeto a aprobación de crédito. Los términos regulares de la cuenta aplican a compras fuera de promoción; para cuentas nuevas al 07/31/2025 la tasa APR de compra es 34.99%, la APR de penalización 39.99% y el cargo mínimo por interés $2. Lacks puede modificar o descontinuar esta oferta en cualquier momento."}},{"id":"synchrony-0-48","kind":"open-end-promotional-credit","provider":"Synchrony","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","apr":0,"termMonths":48,"minimumPurchase":4200,"channel":"in-store","calculationMode":"not-published","paymentCalculationEnabled":false,"headline":{"en":"0% APR for 48 months","es":"0% APR por 48 meses"},"detail":{"en":"On qualifying in-store purchases of $4,200 or more with the Lacks Furniture Synchrony HOME Credit Card. Equal monthly payments required. A minimum purchase and a down payment, plus tax and delivery fee, are required. The advertised purchase minimum must be met on one receipt; discounts may reduce the purchase below it.","es":"En compras en tienda que califiquen de $4,200 o más con la tarjeta Lacks Furniture Synchrony HOME. Se requieren pagos mensuales iguales. Se requiere una compra mínima y un enganche, más impuestos y cargo de entrega. El mínimo de compra anunciado debe cumplirse en un solo recibo; los descuentos pueden reducir la compra por debajo del mínimo."},"disclosure":{"en":"Subject to credit approval. No interest is charged on the promotional purchase. Regular account terms apply to non-promo purchases; for new accounts as of 07/31/2025 the purchase APR is 34.99%, penalty APR 39.99%, minimum interest charge $2.","es":"Sujeto a aprobación de crédito. No se cobra interés en la compra promocional. Los términos regulares de la cuenta aplican a compras fuera de promoción; para cuentas nuevas al 07/31/2025 la tasa APR de compra es 34.99%, la APR de penalización 39.99% y el cargo mínimo por interés $2."}},{"id":"lacks-in-house","kind":"closed-end-installment","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Lacks In-House Credit","es":"Crédito Interno de Lacks"},"detail":{"en":"Installment contracts may be available from 6–36 months for qualifying customers, with in-house approvals by Lacks' own credit team. Purchases may also qualify for promotional pricing. Subject to Lacks approval and applicable offer terms.","es":"Para clientes que califiquen, puede haber contratos a plazos de 6 a 36 meses, con aprobación interna del propio equipo de crédito de Lacks. Las compras también pueden calificar para precios promocionales. Sujeto a la aprobación de Lacks y a los términos de la oferta aplicable."},"disclosure":{"en":"Availability, terms, and promotional pricing are confirmed by Lacks in store.","es":"La disponibilidad, los términos y los precios promocionales los confirma Lacks en tienda."}},{"id":"lease-to-own","kind":"lease-to-own","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Lease-to-own","es":"Arrendamiento con opción a compra"},"detail":{"en":"Lease-to-own is available. Program details, costs, eligibility, and ownership terms are confirmed in store.","es":"El arrendamiento con opción a compra está disponible. Los detalles del programa, costos, elegibilidad y términos de propiedad se confirman en tienda."}},{"id":"build-my-credit","kind":"credit-builder","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Build My Credit","es":"Build My Credit"},"detail":{"en":"An available path for customers with little or no credit history. Program details are confirmed in store.","es":"Una opción disponible para clientes con poco o ningún historial de crédito. Los detalles del programa se confirman en tienda."}},{"id":"mexico-in-house","kind":"closed-end-installment","provider":"Lacks","presentationScenario":"mexico-delivery","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/faq","apr":24,"termMonths":24,"paymentCalculationEnabled":false,"headline":{"en":"Purchasing for delivery to Mexico?","es":"¿Compras para entrega en México?"},"detail":{"en":"An optional program for customers purchasing for delivery to Mexico: Lacks in-house credit for up to 24 months with a maximum contract APR of 24% (which may vary). Requirements currently include two official IDs, three personal references, and income verification.","es":"Un programa opcional para clientes que compran para entrega en México: crédito interno de Lacks hasta por 24 meses con un interés máximo del contrato de 24% APR (mismo que puede variar). Los requisitos actuales incluyen dos identificaciones oficiales, 3 referencias personales y verificación de ingresos."},"representativeExample":{"en":"Lacks' published example: $999 financed for 24 months at 24% APR equals 24 monthly payments of $52.82.","es":"Ejemplo publicado por Lacks: $999 financiados durante 24 meses con 24% APR tendrán 24 pagos mensuales de $52.82."},"disclosure":{"en":"For purchases intended for delivery to Mexico, ask a Lacks specialist to confirm current details and requirements.","es":"Para compras destinadas a entrega en México, consulta con un especialista de Lacks para confirmar los detalles y requisitos actuales."}}]}}</t>
+          <t>{"financing":{"enabled":true,"experience":"payment-choice","offerVersion":"2026-07-30a","verifiedAt":"2026-07-31T16:43:00-05:00","maxAgeDays":7,"sourceUrl":"https://www.lacks.com/financing","applicationUrl":"https://www.lacks.com/credit-application","mexicoInfoUrl":"https://www.lacks.com/faq","mexicoApplicationUrl":{"url":"https://www.lacks.com/mexican-credit-application","verified":false,"note":"Published in Lacks' FAQ but returned 404 on 2026-07-30. Do not render as a link until it resolves; the Mexico card links to mexicoInfoUrl."},"savingsPassPolicy":"specialist_confirm","exactPromotionsEnabled":false,"esReviewStatus":"pending-native-legal-review","allowedSourceHosts":["lacks.com","www.lacks.com","synchrony.com","www.synchrony.com","mysynchrony.com"],"copy":{"eyebrow":{"en":"LACKS PAYMENT CHOICE","es":"OPCIONES DE PAGO LACKS"},"headline":{"en":"Better sleep. More ways to bring it home.","es":"Duerme mejor. Más opciones para llevarlo a casa."},"body":{"en":"Explore promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Options are subject to terms and approval.","es":"Explora financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. Las opciones están sujetas a términos y aprobación."},"cta":{"en":"Explore payment options","es":"Explorar opciones de pago"},"welcomeTagline":{"en":"Flexible ways to bring better sleep home.","es":"Formas flexibles de llevar mejor descanso a casa."},"welcomeSupport":{"en":"Explore payment options after finding your strongest mattress matches.","es":"Explora opciones de pago después de encontrar tus mejores opciones de colchón."},"resultsLead":{"en":"Your strongest mattress match may have more than one way to bring it home.","es":"Tu mejor opción de colchón puede tener más de una forma de llegar a casa."},"resultsAsk":{"en":"Plan the conversation","es":"Planear la conversación"},"fitFirst":{"en":"Your matches are based on sleep fit — never on payment method.","es":"Tus opciones se basan en tu descanso — nunca en la forma de pago."},"drawerTitle":{"en":"Ways to bring it home","es":"Formas de llevarlo a casa"},"drawerBody":{"en":"This recommendation is based on your sleep fit. When you're ready, Lacks offers more than one way to bring it home.","es":"Esta recomendación se basa en tu descanso. Cuando estés listo, Lacks ofrece más de una forma de llevarlo a casa."},"drawerMark":{"en":"Plan the conversation","es":"Planear la conversación"},"sleepSystemGuidance":{"en":"Build the sleep setup that fits you first. Your Lacks specialist can then review current payment options for the complete plan.","es":"Primero arma el sistema de sueño que te quede bien. Después, tu especialista de Lacks puede revisar las opciones de pago actuales para el plan completo."},"handoffHeadline":{"en":"Your Sleep Plan. Your Payment Choices.","es":"Tu Plan de Sueño. Tus Opciones de Pago."},"handoffPrivate":{"en":"Continue on your phone — scan to open Lacks' official financing page.","es":"Continúa desde tu teléfono — escanea para abrir la página oficial de financiamiento de Lacks."},"agendaPrompt":{"en":"As you review these together, mark any options the customer wants to discuss.","es":"Mientras revisan estas opciones juntos, marca las opciones de pago que el cliente quiera conversar."},"agendaMark":{"en":"Add to discussion","es":"Agregar a la conversación"},"agendaMarked":{"en":"Added to discussion","es":"Agregado a la conversación"},"agendaEmpty":{"en":"No options are marked yet.","es":"Todavía no hay opciones de pago marcadas."},"agendaConsequence":{"en":"Use this agenda to guide the conversation together. Nothing is submitted and no application is started.","es":"Usen esta agenda para guiar la conversación juntos. No se envía nada y no se inicia ninguna solicitud."},"agendaChange":{"en":"Change discussion agenda","es":"Cambiar agenda de conversación"},"agendaNotNow":{"en":"Not right now","es":"Ahora no"},"agendaDismissed":{"en":"No options marked for review right now.","es":"No hay opciones de pago marcadas para revisar por ahora."},"agendaDone":{"en":"Done","es":"Listo"},"interestMarkedAnnounce":{"en":"Added to the discussion. Nothing is submitted and no application is started.","es":"Agregado a la conversación. No se envía nada y no se inicia ninguna solicitud."},"interestNotNowAnnounce":{"en":"Not right now selected. You can change this choice.","es":"Se seleccionó 'Ahora no'. Puedes cambiar esta opción."},"interestClearedAnnounce":{"en":"Selection cleared. Choose again when you're ready.","es":"Se borró la selección. Elige de nuevo cuando quieras."},"staleNotice":{"en":"Current payment options are available from your Lacks specialist.","es":"Tu especialista de Lacks tiene las opciones de pago actuales."},"staleAnnouncement":{"en":"Exact rates and terms are not shown right now. Your Lacks specialist can confirm current payment options in store.","es":"Las tasas y los plazos exactos no se muestran en este momento. Tu especialista de Lacks puede confirmar las opciones de pago actuales en tienda."},"externalNotice":{"en":"Opens lacks.com — a separate site governed by its own terms and privacy policy.","es":"Abre lacks.com — un sitio aparte, regido por sus propios términos y política de privacidad."},"emailHeading":{"en":"Payment options","es":"Opciones de pago"},"emailBody":{"en":"You explored Lacks Payment Choice: promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Final pricing, eligibility, terms, and approval are confirmed by Lacks.","es":"Exploraste las Opciones de Pago Lacks: financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. El precio final, la elegibilidad, los términos y la aprobación los confirma Lacks."},"emailBodyAvailable":{"en":"Lacks Payment Choice offers more than one way to bring it home: promotional financing, Lacks In-House Credit, lease-to-own, and Build My Credit. Final pricing, eligibility, terms, and approval are confirmed by Lacks.","es":"Las Opciones de Pago Lacks ofrecen más de una forma de llevarlo a casa: financiamiento promocional, Crédito Interno de Lacks, arrendamiento con opción a compra y Build My Credit. El precio final, la elegibilidad, los términos y la aprobación los confirma Lacks."},"disclosureFooter":{"en":"All payment options are subject to terms and approval. Advertised purchase minimums, rates, and terms are set by Lacks and its financing partners and may change or end at any time. Your Lacks specialist confirms current details in store.","es":"Todas las opciones de pago están sujetas a términos y aprobación. Los mínimos de compra, tasas y plazos anunciados los establecen Lacks y sus socios financieros y pueden cambiar o terminar en cualquier momento. Tu especialista de Lacks confirma los detalles vigentes en tienda."},"prequalNote":{"en":"See if you prequalify on Lacks' official financing page — prequalification is not approval.","es":"Consulta si precalificas en la página oficial de financiamiento de Lacks — precalificar no es una aprobación."}},"plans":[{"id":"synchrony-9-99-72","kind":"open-end-promotional-credit","provider":"Synchrony","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","apr":9.99,"termMonths":72,"minimumPurchase":500,"channel":"per-current-source","calculationMode":"published-fixed-factor","paymentCalculationEnabled":false,"headline":{"en":"9.99% APR for 72 months","es":"9.99% APR por 72 meses"},"detail":{"en":"On qualifying purchases of $500 or more with the Lacks Furniture Synchrony HOME Credit Card. Fixed monthly payments required. Interest is charged from the purchase date at the reduced APR. The advertised purchase minimum must be met on one receipt; discounts may reduce the purchase below it.","es":"En compras que califiquen de $500 o más con la tarjeta Lacks Furniture Synchrony HOME. Se requieren pagos mensuales fijos. Se cobra interés desde la fecha de compra a la tasa APR reducida. El mínimo de compra anunciado debe cumplirse en un solo recibo; los descuentos pueden reducir la compra por debajo del mínimo."},"disclosure":{"en":"Subject to credit approval. Regular account terms apply to non-promo purchases; for new accounts as of 07/31/2025 the purchase APR is 34.99%, penalty APR 39.99%, minimum interest charge $2. Lacks may alter or discontinue this offer at any time.","es":"Sujeto a aprobación de crédito. Los términos regulares de la cuenta aplican a compras fuera de promoción; para cuentas nuevas al 07/31/2025 la tasa APR de compra es 34.99%, la APR de penalización 39.99% y el cargo mínimo por interés $2. Lacks puede modificar o descontinuar esta oferta en cualquier momento."}},{"id":"synchrony-0-48","kind":"open-end-promotional-credit","provider":"Synchrony","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","apr":0,"termMonths":48,"minimumPurchase":4200,"channel":"in-store","calculationMode":"not-published","paymentCalculationEnabled":false,"headline":{"en":"0% APR for 48 months","es":"0% APR por 48 meses"},"detail":{"en":"On qualifying in-store purchases of $4,200 or more with the Lacks Furniture Synchrony HOME Credit Card. Equal monthly payments required. A minimum purchase and a down payment, plus tax and delivery fee, are required. The advertised purchase minimum must be met on one receipt; discounts may reduce the purchase below it.","es":"En compras en tienda que califiquen de $4,200 o más con la tarjeta Lacks Furniture Synchrony HOME. Se requieren pagos mensuales iguales. Se requiere una compra mínima y un enganche, más impuestos y cargo de entrega. El mínimo de compra anunciado debe cumplirse en un solo recibo; los descuentos pueden reducir la compra por debajo del mínimo."},"disclosure":{"en":"Subject to credit approval. No interest is charged on the promotional purchase. Regular account terms apply to non-promo purchases; for new accounts as of 07/31/2025 the purchase APR is 34.99%, penalty APR 39.99%, minimum interest charge $2.","es":"Sujeto a aprobación de crédito. No se cobra interés en la compra promocional. Los términos regulares de la cuenta aplican a compras fuera de promoción; para cuentas nuevas al 07/31/2025 la tasa APR de compra es 34.99%, la APR de penalización 39.99% y el cargo mínimo por interés $2."}},{"id":"lacks-in-house","kind":"closed-end-installment","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Lacks In-House Credit","es":"Crédito Interno de Lacks"},"detail":{"en":"Installment contracts may be available from 6–36 months for qualifying customers, with in-house approvals by Lacks' own credit team. Purchases may also qualify for promotional pricing. Subject to Lacks approval and applicable offer terms.","es":"Para clientes que califiquen, puede haber contratos a plazos de 6 a 36 meses, con aprobación interna del propio equipo de crédito de Lacks. Las compras también pueden calificar para precios promocionales. Sujeto a la aprobación de Lacks y a los términos de la oferta aplicable."},"disclosure":{"en":"Availability, terms, and promotional pricing are confirmed by Lacks in store.","es":"La disponibilidad, los términos y los precios promocionales los confirma Lacks en tienda."}},{"id":"lease-to-own","kind":"lease-to-own","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Lease-to-own","es":"Arrendamiento con opción a compra"},"detail":{"en":"Lease-to-own is available. Program details, costs, eligibility, and ownership terms are confirmed in store.","es":"El arrendamiento con opción a compra está disponible. Los detalles del programa, costos, elegibilidad y términos de propiedad se confirman en tienda."}},{"id":"build-my-credit","kind":"credit-builder","provider":"Lacks","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/financing","paymentCalculationEnabled":false,"headline":{"en":"Build My Credit","es":"Build My Credit"},"detail":{"en":"An available path for customers with little or no credit history. Program details are confirmed in store.","es":"Una opción disponible para clientes con poco o ningún historial de crédito. Los detalles del programa se confirman en tienda."}},{"id":"mexico-in-house","kind":"closed-end-installment","provider":"Lacks","presentationScenario":"mexico-delivery","verified":true,"verifiedAt":"2026-07-31T16:43:00-05:00","sourceUrl":"https://www.lacks.com/faq","apr":24,"termMonths":24,"paymentCalculationEnabled":false,"headline":{"en":"Purchasing for delivery to Mexico?","es":"¿Compras para entrega en México?"},"detail":{"en":"An optional program for customers purchasing for delivery to Mexico: Lacks in-house credit for up to 24 months with a maximum contract APR of 24% (which may vary). Requirements currently include two official IDs, three personal references, and income verification.","es":"Un programa opcional para clientes que compran para entrega en México: crédito interno de Lacks hasta por 24 meses con un interés máximo del contrato de 24% APR (mismo que puede variar). Los requisitos actuales incluyen dos identificaciones oficiales, 3 referencias personales y verificación de ingresos."},"representativeExample":{"en":"Lacks' published example: $999 financed for 24 months at 24% APR equals 24 monthly payments of $52.82.","es":"Ejemplo publicado por Lacks: $999 financiados durante 24 meses con 24% APR tendrán 24 pagos mensuales de $52.82."},"disclosure":{"en":"For purchases intended for delivery to Mexico, ask a Lacks specialist to confirm current details and requirements.","es":"Para compras destinadas a entrega en México, consulta con un especialista de Lacks para confirmar los detalles y requisitos actuales."}}]}}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct landing store locations
</commit_message>
<xml_diff>
--- a/incoming/Lacks_Store_Data.xlsx
+++ b/incoming/Lacks_Store_Data.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Store Info" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Brands" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Mattresses" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Accessories" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SalesNotes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Promotions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Quiz" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Store Info" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brands" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mattresses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accessories" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SalesNotes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1180,7 +1180,7 @@
       <c r="BR2" t="inlineStr"/>
       <c r="BS2" t="inlineStr">
         <is>
-          <t>McAllen · Pharr · Harlingen · Brownsville · Rio Grande City · Laredo · Alice · Corpus Christi</t>
+          <t>Brownsville · Laredo · McAllen · Alice · Harlingen · Rio Grande City</t>
         </is>
       </c>
       <c r="BT2" t="inlineStr">

</xml_diff>

<commit_message>
Remove the two zero-scoring quiz questions (12 -> 10, owner ruling)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/incoming/Lacks_Store_Data.xlsx
+++ b/incoming/Lacks_Store_Data.xlsx
@@ -6011,7 +6011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>sleep_quality.poor</t>
+          <t>trigger.pain</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -6275,7 +6275,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>aiming for a real change in nightly rest</t>
+          <t>here to solve a comfort problem</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -6285,7 +6285,7 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
-          <t>buscando un cambio real en el descanso</t>
+          <t>aquí para resolver un problema de comodidad</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>sleep_quality.fair</t>
+          <t>trigger.worn_out</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -6308,7 +6308,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>aiming to sleep noticeably better</t>
+          <t>replacing an old mattress</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -6318,7 +6318,7 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
-          <t>buscando dormir notablemente mejor</t>
+          <t>reemplazando un colchón viejo</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>sleep_quality.okay</t>
+          <t>trigger.moving</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -6341,7 +6341,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>building on what already works</t>
+          <t>furnishing a new space</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -6351,7 +6351,7 @@
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
-          <t>mejorando lo que ya funciona</t>
+          <t>amueblando un espacio nuevo</t>
         </is>
       </c>
     </row>
@@ -6363,7 +6363,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>sleep_quality.well</t>
+          <t>trigger.upgrade</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -6374,7 +6374,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>protecting a setup that already works</t>
+          <t>ready for an upgrade</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -6384,7 +6384,7 @@
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
-          <t>cuidando un descanso que ya funciona</t>
+          <t>buscando una mejora</t>
         </is>
       </c>
     </row>
@@ -6396,7 +6396,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>trigger.pain</t>
+          <t>trigger.browsing</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -6407,7 +6407,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>here to solve a comfort problem</t>
+          <t>exploring options today</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -6417,7 +6417,7 @@
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
-          <t>aquí para resolver un problema de comodidad</t>
+          <t>explorando opciones hoy</t>
         </is>
       </c>
     </row>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>trigger.worn_out</t>
+          <t>sleep_issues.back_pain</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -6440,7 +6440,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>replacing an old mattress</t>
+          <t>test lower-back support carefully</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -6450,7 +6450,7 @@
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
-          <t>reemplazando un colchón viejo</t>
+          <t>probar con cuidado el soporte lumbar</t>
         </is>
       </c>
     </row>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>trigger.moving</t>
+          <t>sleep_issues.hip_pain</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -6473,7 +6473,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>furnishing a new space</t>
+          <t>focus on pressure relief at hips and shoulders</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -6483,7 +6483,7 @@
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
-          <t>amueblando un espacio nuevo</t>
+          <t>enfocarse en aliviar la presión en caderas y hombros</t>
         </is>
       </c>
     </row>
@@ -6495,7 +6495,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>trigger.upgrade</t>
+          <t>sleep_issues.hot</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -6506,7 +6506,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ready for an upgrade</t>
+          <t>prioritize temperature control</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -6516,7 +6516,7 @@
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
-          <t>buscando una mejora</t>
+          <t>priorizar el control de temperatura</t>
         </is>
       </c>
     </row>
@@ -6528,7 +6528,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>trigger.browsing</t>
+          <t>sleep_issues.tossing</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -6539,7 +6539,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>exploring options today</t>
+          <t>notice how easy it is to settle in</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -6549,7 +6549,7 @@
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
-          <t>explorando opciones hoy</t>
+          <t>notar qué tan fácil es acomodarse</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>sleep_issues.back_pain</t>
+          <t>sleep_issues.stiff</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -6572,7 +6572,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>test lower-back support carefully</t>
+          <t>compare alignment and morning comfort</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -6582,7 +6582,7 @@
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
-          <t>probar con cuidado el soporte lumbar</t>
+          <t>comparar la alineación y la comodidad al despertar</t>
         </is>
       </c>
     </row>
@@ -6594,7 +6594,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>sleep_issues.hip_pain</t>
+          <t>sleep_issues.sagging</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -6605,7 +6605,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>focus on pressure relief at hips and shoulders</t>
+          <t>check for durable, consistent support</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -6615,7 +6615,7 @@
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
-          <t>enfocarse en aliviar la presión en caderas y hombros</t>
+          <t>revisar que el soporte sea duradero y consistente</t>
         </is>
       </c>
     </row>
@@ -6627,7 +6627,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>sleep_issues.hot</t>
+          <t>sleep_issues.too_soft</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -6638,7 +6638,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>prioritize temperature control</t>
+          <t>try firmer, more supportive feels</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -6648,7 +6648,7 @@
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr">
         <is>
-          <t>priorizar el control de temperatura</t>
+          <t>probar sensaciones más firmes y con más soporte</t>
         </is>
       </c>
     </row>
@@ -6660,7 +6660,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>sleep_issues.tossing</t>
+          <t>sleep_issues.none</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -6669,21 +6669,13 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>notice how easy it is to settle in</t>
-        </is>
-      </c>
+      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>notar qué tan fácil es acomodarse</t>
-        </is>
-      </c>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6693,7 +6685,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>sleep_issues.stiff</t>
+          <t>sleep_position.side</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -6704,7 +6696,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>compare alignment and morning comfort</t>
+          <t>prioritize shoulder and hip cushioning</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -6714,7 +6706,7 @@
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
-          <t>comparar la alineación y la comodidad al despertar</t>
+          <t>priorizar el acolchado de hombros y caderas</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6718,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>sleep_issues.sagging</t>
+          <t>sleep_position.back</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -6737,7 +6729,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>check for durable, consistent support</t>
+          <t>look for even lumbar support</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -6747,7 +6739,7 @@
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
-          <t>revisar que el soporte sea duradero y consistente</t>
+          <t>buscar soporte lumbar uniforme</t>
         </is>
       </c>
     </row>
@@ -6759,7 +6751,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>sleep_issues.too_soft</t>
+          <t>sleep_position.stomach</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -6770,7 +6762,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>try firmer, more supportive feels</t>
+          <t>keep the midsection supported</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -6780,7 +6772,7 @@
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
-          <t>probar sensaciones más firmes y con más soporte</t>
+          <t>mantener la zona media con soporte</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6784,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>sleep_issues.none</t>
+          <t>sleep_position.combo</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -6801,13 +6793,21 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>notice ease of movement between positions</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>notar la facilidad para cambiar de posición</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6817,7 +6817,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>sleep_position.side</t>
+          <t>sleep_position.no_idea</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -6828,7 +6828,7 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>prioritize shoulder and hip cushioning</t>
+          <t>compare a few different feels to find a starting point</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -6838,7 +6838,7 @@
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
-          <t>priorizar el acolchado de hombros y caderas</t>
+          <t>comparar varias sensaciones para encontrar un punto de partida</t>
         </is>
       </c>
     </row>
@@ -6850,7 +6850,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>sleep_position.back</t>
+          <t>health_conditions.nerve_pain</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -6861,7 +6861,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>look for even lumbar support</t>
+          <t>compare gentle, even pressure relief</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -6871,7 +6871,7 @@
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
-          <t>buscar soporte lumbar uniforme</t>
+          <t>comparar un alivio de presión suave y uniforme</t>
         </is>
       </c>
     </row>
@@ -6883,7 +6883,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>sleep_position.stomach</t>
+          <t>health_conditions.allergies</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -6894,7 +6894,7 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>keep the midsection supported</t>
+          <t>ask about washable and protective covers</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -6904,7 +6904,7 @@
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
-          <t>mantener la zona media con soporte</t>
+          <t>preguntar por fundas lavables y protectoras</t>
         </is>
       </c>
     </row>
@@ -6916,7 +6916,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>sleep_position.combo</t>
+          <t>health_conditions.snoring</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -6927,7 +6927,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>notice ease of movement between positions</t>
+          <t>test head-of-bed elevation on an adjustable base</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -6937,7 +6937,7 @@
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
-          <t>notar la facilidad para cambiar de posición</t>
+          <t>probar la elevación de la cabecera en una base ajustable</t>
         </is>
       </c>
     </row>
@@ -6949,7 +6949,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>sleep_position.no_idea</t>
+          <t>health_conditions.reflux</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -6960,7 +6960,7 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>compare a few different feels to find a starting point</t>
+          <t>notice how a raised upper body feels</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
@@ -6970,7 +6970,7 @@
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
-          <t>comparar varias sensaciones para encontrar un punto de partida</t>
+          <t>notar cómo se siente el torso elevado</t>
         </is>
       </c>
     </row>
@@ -6982,7 +6982,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>health_conditions.nerve_pain</t>
+          <t>health_conditions.extra_support</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -6993,7 +6993,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>compare gentle, even pressure relief</t>
+          <t>prioritize reinforced, sturdy support</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -7003,7 +7003,7 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
-          <t>comparar un alivio de presión suave y uniforme</t>
+          <t>priorizar un soporte reforzado y resistente</t>
         </is>
       </c>
     </row>
@@ -7015,7 +7015,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>health_conditions.allergies</t>
+          <t>health_conditions.getting_older</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -7026,7 +7026,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>ask about washable and protective covers</t>
+          <t>compare ease of getting in and out of bed</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -7036,7 +7036,7 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr">
         <is>
-          <t>preguntar por fundas lavables y protectoras</t>
+          <t>comparar la facilidad para acostarse y levantarse</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7048,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>health_conditions.snoring</t>
+          <t>health_conditions.none</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -7057,21 +7057,13 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>test head-of-bed elevation on an adjustable base</t>
-        </is>
-      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>probar la elevación de la cabecera en una base ajustable</t>
-        </is>
-      </c>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7081,7 +7073,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>health_conditions.reflux</t>
+          <t>temperature.hot</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -7092,7 +7084,7 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>notice how a raised upper body feels</t>
+          <t>compare cooling covers and airflow</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
@@ -7102,7 +7094,7 @@
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
-          <t>notar cómo se siente el torso elevado</t>
+          <t>comparar fundas frescas y ventilación</t>
         </is>
       </c>
     </row>
@@ -7114,7 +7106,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>health_conditions.extra_support</t>
+          <t>temperature.comfortable</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -7123,21 +7115,13 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>prioritize reinforced, sturdy support</t>
-        </is>
-      </c>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>priorizar un soporte reforzado y resistente</t>
-        </is>
-      </c>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7147,7 +7131,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>health_conditions.getting_older</t>
+          <t>temperature.cold</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -7158,7 +7142,7 @@
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>compare ease of getting in and out of bed</t>
+          <t>notice warmth and cozier surface feels</t>
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
@@ -7168,7 +7152,7 @@
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr">
         <is>
-          <t>comparar la facilidad para acostarse y levantarse</t>
+          <t>notar calidez y superficies más acogedoras</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7164,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>health_conditions.none</t>
+          <t>temperature.opposite</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -7189,133 +7173,17 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>compare temperature balance for two sleepers</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>consultation</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>temperature.hot</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>compare cooling covers and airflow</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>comparar fundas frescas y ventilación</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>consultation</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>temperature.comfortable</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>consultation</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>temperature.cold</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>notice warmth and cozier surface feels</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>notar calidez y superficies más acogedoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>consultation</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>temperature.opposite</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>compare temperature balance for two sleepers</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>comparar el equilibrio de temperatura para dos personas</t>
         </is>
@@ -7373,7 +7241,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"quiz":{"questions":[{"id":"sleep_quality","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"How well do you sleep right now?","es":"¿Qué tan bien duermes actualmente?"},"helpText":{"en":"Be honest. It helps us solve the real problem, not guess.","es":"Sé honesto — podemos ayudarte de cualquier manera"},"type":"single","options":[{"id":"poor","label":{"en":"Poorly","es":"Mal"},"icon":"stiff","sublabel":{"en":"Restless, waking often","es":"Inquieto, despertando seguido"},"scores":{}},{"id":"fair","label":{"en":"Not Great","es":"No Muy Bien"},"icon":"combo","sublabel":{"en":"Could be a lot better","es":"Podría ser mucho mejor"},"scores":{}},{"id":"okay","label":{"en":"Okay","es":"Más o Menos"},"icon":"smile","sublabel":{"en":"Mostly fine","es":"Generalmente bien"},"scores":{}},{"id":"well","label":{"en":"Pretty Well","es":"Bastante Bien"},"icon":"check","sublabel":{"en":"Usually rested","es":"Generalmente descansado"},"scores":{}}]},{"id":"trigger","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What can we help you with today?","es":"¿En qué te podemos ayudar hoy?"},"helpText":{"en":"No pressure — this just helps your specialist focus on what matters to you.","es":"Sin presión — esto ayuda a tu especialista a enfocarse en lo que te importa."},"type":"single","options":[{"id":"pain","label":{"en":"Back or Body Pain","es":"Dolor de Espalda o Cuerpo"},"icon":"spine","sublabel":{"en":"Current mattress is hurting me","es":"Mi colchón actual me lastima"},"scores":{}},{"id":"worn_out","label":{"en":"Old Mattress","es":"Colchón Viejo"},"icon":"sagging","sublabel":{"en":"Time for an upgrade","es":"Es hora de un cambio"},"scores":{}},{"id":"moving","label":{"en":"Moving or New Space","es":"Mudanza o Espacio Nuevo"},"icon":"family","sublabel":{"en":"New home, new bed","es":"Casa nueva, cama nueva"},"scores":{}},{"id":"upgrade","label":{"en":"Just Upgrading","es":"Mejorando"},"icon":"cloud","sublabel":{"en":"Ready for something better","es":"Listo para algo mejor"},"scores":{}},{"id":"browsing","label":{"en":"Just Browsing","es":"Solo Explorando"},"icon":"smile","sublabel":{"en":"Getting ideas, no rush","es":"Sin prisa, juntando ideas"},"scores":{}}]},{"id":"mattress_size","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What size mattress are you looking for?","es":"¿Qué tamaño de colchón buscas?"},"helpText":{"en":"So every mattress we show actually fits your space.","es":"Nos aseguraremos de que las recomendaciones se ajusten a tu espacio"},"type":"single","options":[{"id":"twin","label":{"en":"Twin","es":"Twin"},"icon":"solo","sublabel":{"en":"Kids or tight spaces","es":"Niños o espacios pequeños"},"scores":{}},{"id":"twin_xl","label":{"en":"Twin XL","es":"Twin XL"},"icon":"solo","sublabel":{"en":"Extra length, single sleeper","es":"Largo extra, una persona"},"scores":{}},{"id":"full","label":{"en":"Full","es":"Full"},"icon":"solo","sublabel":{"en":"Solo or cozy pair","es":"Solo o pareja cómoda"},"scores":{}},{"id":"queen","label":{"en":"Queen","es":"Queen"},"icon":"partner","sublabel":{"en":"Most popular size","es":"El tamaño más popular"},"scores":{}},{"id":"king","label":{"en":"King","es":"King"},"icon":"family","sublabel":{"en":"Maximum space","es":"Espacio máximo"},"scores":{}},{"id":"cal_king","label":{"en":"Cal King","es":"Cal King"},"icon":"family","sublabel":{"en":"Extra length","es":"Largo extra"},"scores":{}}]},{"id":"partner_sleep","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Who's sharing the bed with you?","es":"¿Quién comparte la cama contigo?"},"helpText":{"en":"Who shares your bed shapes which features matter most.","es":"Esto determina qué características importan más"},"type":"single","options":[{"id":"solo","label":{"en":"Solo Sleeper","es":"Duermo Solo"},"icon":"solo","sublabel":{"en":"Just me","es":"Solo yo"},"scores":{}},{"id":"partner","label":{"en":"With a Partner","es":"Con Pareja"},"icon":"partner","sublabel":{"en":"Sharing the bed","es":"Compartimos la cama"},"scores":{"motionIsolation":2}},{"id":"family","label":{"en":"Family Bed","es":"Cama Familiar"},"icon":"family","sublabel":{"en":"Kids, pets, or both","es":"Niños, mascotas, o ambos"},"scores":{"durability":2,"motionIsolation":1}}]},{"id":"partner_disturbance","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Does your partner's movement wake you up?","es":"¿El movimiento de tu pareja te despierta?"},"helpText":{"en":"Motion isolation is one of the first upgrades you'll feel.","es":"El aislamiento de movimiento es una de las mayores mejoras en un colchón nuevo"},"type":"single","skipIf":{"question":"partner_sleep","answer":"solo"},"options":[{"id":"yes_often","label":{"en":"Yes, Often","es":"Sí, Seguido"},"icon":"motion","sublabel":{"en":"Every movement wakes me","es":"Cada movimiento me despierta"},"scores":{"motionIsolation":4,"hybrid":3,"memory":2}},{"id":"sometimes","label":{"en":"Sometimes","es":"A Veces"},"icon":"combo","sublabel":{"en":"Bigger movements bother me","es":"Los movimientos grandes me molestan"},"scores":{"motionIsolation":3,"hybrid":2}},{"id":"rarely","label":{"en":"Rarely","es":"Rara Vez"},"icon":"check","sublabel":{"en":"Light sleeper but mostly fine","es":"Sueño ligero pero generalmente bien"},"scores":{"motionIsolation":1}},{"id":"not_applicable","label":{"en":"Doesn't Apply","es":"No Aplica"},"icon":"solo","sublabel":{"en":"I sleep alone","es":"Duermo solo"},"scores":{}}]},{"id":"sleep_position","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"How do you usually sleep?","es":"¿Cómo duermes normalmente?"},"helpText":{"en":"Your sleep position is the biggest clue to the support you need.","es":"Piensa en cómo terminas naturalmente"},"type":"single","options":[{"id":"side","label":{"en":"Side Sleeper","es":"De Lado"},"icon":"side","sublabel":{"en":"Curled up","es":"Acurrucado"},"scores":{"plush":2,"pressureRelief":2,"soft":1}},{"id":"back","label":{"en":"Back Sleeper","es":"Boca Arriba"},"icon":"back","sublabel":{"en":"Flat on back","es":"Acostado de espalda"},"scores":{"support":2,"medium":2,"zoned":1}},{"id":"stomach","label":{"en":"Stomach Sleeper","es":"Boca Abajo"},"icon":"stomach","sublabel":{"en":"Face down","es":"Boca abajo"},"scores":{"firm":2,"support":1}},{"id":"combo","label":{"en":"Combination","es":"Combinación"},"icon":"combo","sublabel":{"en":"Move around","es":"Me muevo mucho"},"scores":{"medium":2,"responsive":2}},{"id":"no_idea","label":{"en":"Not Sure","es":"No Estoy Seguro"},"icon":"question","sublabel":{"en":"I wake up in weird positions","es":"Me despierto en posiciones raras"},"scores":{"medium":2,"responsive":2}}]},{"id":"body_type","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"What weight range should this mattress support?","es":"¿Qué rango de peso debe soportar este colchón?"},"helpText":{"en":"This helps us account for cushioning, support, and durability.","es":"Esto nos ayuda a considerar la amortiguación, el soporte y la durabilidad."},"type":"single","options":[{"id":"petite","label":{"en":"Under 130 lbs","es":"Menos de 130 lbs"},"icon":"cloud","sublabel":{"en":"Light support","es":"Soporte ligero"},"scores":{"plush":2,"soft":1}},{"id":"average","label":{"en":"130 to 200 lbs","es":"130 a 200 lbs"},"icon":"weight","sublabel":{"en":"Standard support","es":"Soporte estándar"},"scores":{"medium":2}},{"id":"athletic","label":{"en":"200 to 230 lbs","es":"200 a 230 lbs"},"icon":"support","sublabel":{"en":"Medium-firm support","es":"Soporte medio-firme"},"scores":{"support":2,"medium":1,"responsive":1}},{"id":"plus","label":{"en":"Over 230 lbs","es":"Más de 230 lbs"},"icon":"support","sublabel":{"en":"Maximum support","es":"Soporte máximo"},"scores":{"firm":2,"support":3,"hybrid":2,"durability":2}},{"id":"different","label":{"en":"Different weight ranges","es":"Rangos de peso diferentes"},"icon":"partner","sublabel":{"en":"Sleepers fall into different ranges","es":"Los durmientes están en rangos diferentes"},"scores":{"medium":2,"support":1,"motionIsolation":2},"hideIf":{"question":"partner_sleep","answer":"solo"}}],"copyVariants":[{"when":{"question":"partner_sleep","answerIn":["partner","family"]},"question":{"en":"What weight range should we match for the sleeper who needs more support?","es":"¿Para qué rango de peso debemos ajustar, según quien necesite más soporte?"},"helpText":{"en":"If you fall into different ranges, choose “Different weight ranges.”","es":"Si están en rangos diferentes, elige “Rangos de peso diferentes”."}}]},{"id":"temperature","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"How do you sleep temperature-wise?","es":"¿Cómo duermes en cuanto a temperatura?"},"helpText":{"en":"Sleeping hot or cold is an easy fix with the right materials.","es":"La regulación de temperatura es clave para un sueño profundo"},"type":"single","options":[{"id":"hot","label":{"en":"I Sleep Hot","es":"Duermo con Calor"},"icon":"flame","sublabel":{"en":"Night sweats, kick off covers","es":"Sudores nocturnos, quito las cobijas"},"scores":{"cooling":3,"hybrid":2}},{"id":"comfortable","label":{"en":"I'm Comfortable","es":"Estoy Cómodo"},"icon":"smile","sublabel":{"en":"No temperature issues","es":"Sin problemas de temperatura"},"scores":{}},{"id":"cold","label":{"en":"I Sleep Cold","es":"Duermo con Frío"},"icon":"snowflake","sublabel":{"en":"Need blankets to warm up","es":"Necesito cobijas para calentarme"},"scores":{"memory":1,"plush":1}},{"id":"opposite","label":{"en":"We're Opposite","es":"Somos Opuestos"},"icon":"hotcold","sublabel":{"en":"One hot, one cold","es":"Uno con calor, otro con frío"},"scores":{"cooling":2,"hybrid":1},"hideIf":{"question":"partner_sleep","answer":"solo"}}]},{"id":"firmness","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"What firmness level do you prefer?","es":"¿Qué nivel de firmeza prefieres?"},"helpText":{"en":"No wrong answer here, just slide to what feels best.","es":"Desliza a tu comodidad ideal"},"type":"slider","min":1,"max":10,"defaultValue":5,"labels":[{"en":"Soft — Sink right in","es":"Suave — Hundirse"},{"en":"Medium","es":"Medio"},{"en":"Firm — Solid support","es":"Firme — Soporte sólido"}]},{"id":"current_mattress_age","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"How old is your current mattress?","es":"¿Cuántos años tiene tu colchón actual?"},"helpText":{"en":"Most mattresses lose their support after about 8 years.","es":"La mayoría de los colchones duran 7–10 años"},"type":"single","options":[{"id":"under_2","label":{"en":"Less Than 2 Years","es":"Menos de 2 Años"},"icon":"check","sublabel":{"en":"Pretty new","es":"Bastante nuevo"},"scores":{}},{"id":"three_seven","label":{"en":"3 to 7 Years","es":"3 a 7 Años"},"icon":"combo","sublabel":{"en":"Middle of its life","es":"A mitad de su vida"},"scores":{}},{"id":"eight_fifteen","label":{"en":"8 to 15 Years","es":"8 a 15 Años"},"icon":"aging","sublabel":{"en":"Past its prime","es":"Ya pasó su mejor momento"},"scores":{}},{"id":"fifteen_plus","label":{"en":"Over 15 Years","es":"Más de 15 Años"},"icon":"sagging","sublabel":{"en":"Long overdue","es":"Ya era hora"},"scores":{}},{"id":"not_sure","label":{"en":"Not Sure","es":"No Estoy Seguro"},"icon":"question","sublabel":{"en":"Can't remember","es":"No recuerdo"},"scores":{}}]},{"id":"sleep_issues","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Any issues with your current mattress?","es":"¿Algún problema con tu colchón actual?"},"helpText":{"en":"Tap anything you've noticed. Each one points us toward a fix.","es":"Toca las que apliquen"},"type":"multiple","options":[{"id":"back_pain","label":{"en":"Back Pain","es":"Dolor de Espalda"},"icon":"spine","sublabel":{"en":"Lower or upper back","es":"Espalda baja o alta"},"scores":{"support":3,"zoned":2,"firm":1}},{"id":"hip_pain","label":{"en":"Hip or Shoulder Pain","es":"Dolor de Cadera u Hombro"},"icon":"pressure","sublabel":{"en":"Pressure points","es":"Puntos de presión"},"scores":{"pressureRelief":3,"plush":2}},{"id":"hot","label":{"en":"Sleeping Too Hot","es":"Mucho Calor al Dormir"},"icon":"flame","sublabel":{"en":"Night sweats, overheating","es":"Sudores nocturnos, sobrecalentamiento"},"scores":{"cooling":3,"hybrid":2}},{"id":"tossing","label":{"en":"Tossing &amp; Turning","es":"Dando Vueltas"},"icon":"combo","sublabel":{"en":"Can't get comfortable","es":"No encuentro comodidad"},"scores":{"comfort":2,"medium":1}},{"id":"stiff","label":{"en":"Waking Up Stiff or Sore","es":"Despertar Rígido o Adolorido"},"icon":"stiff","sublabel":{"en":"Morning aches","es":"Dolores matutinos"},"scores":{"pressureRelief":2,"comfort":2}},{"id":"sagging","label":{"en":"Mattress Sagging","es":"Colchón Hundido"},"icon":"sagging","sublabel":{"en":"Dips or indentations","es":"Hundimientos"},"scores":{"durability":2,"quality":2}},{"id":"too_soft","label":{"en":"Mattress Too Soft","es":"Colchón Muy Suave"},"icon":"couch","sublabel":{"en":"Sinking in too much","es":"Me hundo demasiado"},"scores":{"firm":3,"support":2}},{"id":"none","label":{"en":"No Major Issues","es":"Sin Problemas Grandes"},"icon":"check","sublabel":{"en":"Just time for an upgrade","es":"Solo es hora de un cambio"},"scores":{"comfort":1,"quality":1,"durable":1}}]},{"id":"health_conditions","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Anything else going on that affects your sleep?","es":"¿Algo más que afecte tu sueño?"},"helpText":{"en":"Tap any that apply. A few of these change what we'd suggest.","es":"Toca las que apliquen"},"type":"multiple","options":[{"id":"nerve_pain","label":{"en":"Nerve Pain or Tingling","es":"Dolor Nervioso u Hormigueo"},"icon":"lightning","sublabel":{"en":"Shooting pain, numbness","es":"Dolor punzante, entumecimiento"},"scores":{"support":3,"firm":2,"zoned":2}},{"id":"allergies","label":{"en":"Allergies","es":"Alergias"},"icon":"sneeze","sublabel":{"en":"Dust, sneezing, stuffy","es":"Polvo, estornudos, congestión"},"scores":{"hypoallergenic":3}},{"id":"snoring","label":{"en":"Snoring or Sleep Apnea","es":"Ronquidos o Apnea del Sueño"},"icon":"snore","sublabel":{"en":"You or your partner","es":"Tú o tu pareja"},"scores":{"adjustable":3}},{"id":"reflux","label":{"en":"Acid Reflux / Heartburn","es":"Reflujo Ácido / Acidez"},"icon":"flame","sublabel":{"en":"Burns when lying down","es":"Arde al acostarse"},"scores":{"adjustable":3}},{"id":"extra_support","label":{"en":"Need Extra Support","es":"Necesito Soporte Extra"},"icon":"weight","sublabel":{"en":"Larger build or heavier weight","es":"Complexión grande o peso mayor"},"scores":{"support":3,"firm":2,"durable":3}},{"id":"getting_older","label":{"en":"Changing Needs","es":"Necesidades Cambiantes"},"icon":"aging","sublabel":{"en":"Looking for gentler support","es":"Buscando soporte más suave"},"scores":{"support":2,"comfort":2,"pressureRelief":1}},{"id":"none","label":{"en":"None of These","es":"Ninguno de Estos"},"icon":"check","sublabel":{"en":"I'm good","es":"Estoy bien"},"scores":{}}]}]}}</t>
+          <t>{"quiz":{"questions":[{"id":"trigger","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What can we help you with today?","es":"¿En qué te podemos ayudar hoy?"},"helpText":{"en":"No pressure — this just helps your specialist focus on what matters to you.","es":"Sin presión — esto ayuda a tu especialista a enfocarse en lo que te importa."},"type":"single","options":[{"id":"pain","label":{"en":"Back or Body Pain","es":"Dolor de Espalda o Cuerpo"},"icon":"spine","sublabel":{"en":"Current mattress is hurting me","es":"Mi colchón actual me lastima"},"scores":{}},{"id":"worn_out","label":{"en":"Old Mattress","es":"Colchón Viejo"},"icon":"sagging","sublabel":{"en":"Time for an upgrade","es":"Es hora de un cambio"},"scores":{}},{"id":"moving","label":{"en":"Moving or New Space","es":"Mudanza o Espacio Nuevo"},"icon":"family","sublabel":{"en":"New home, new bed","es":"Casa nueva, cama nueva"},"scores":{}},{"id":"upgrade","label":{"en":"Just Upgrading","es":"Mejorando"},"icon":"cloud","sublabel":{"en":"Ready for something better","es":"Listo para algo mejor"},"scores":{}},{"id":"browsing","label":{"en":"Just Browsing","es":"Solo Explorando"},"icon":"smile","sublabel":{"en":"Getting ideas, no rush","es":"Sin prisa, juntando ideas"},"scores":{}}]},{"id":"mattress_size","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What size mattress are you looking for?","es":"¿Qué tamaño de colchón buscas?"},"helpText":{"en":"So every mattress we show actually fits your space.","es":"Nos aseguraremos de que las recomendaciones se ajusten a tu espacio"},"type":"single","options":[{"id":"twin","label":{"en":"Twin","es":"Twin"},"icon":"solo","sublabel":{"en":"Kids or tight spaces","es":"Niños o espacios pequeños"},"scores":{}},{"id":"twin_xl","label":{"en":"Twin XL","es":"Twin XL"},"icon":"solo","sublabel":{"en":"Extra length, single sleeper","es":"Largo extra, una persona"},"scores":{}},{"id":"full","label":{"en":"Full","es":"Full"},"icon":"solo","sublabel":{"en":"Solo or cozy pair","es":"Solo o pareja cómoda"},"scores":{}},{"id":"queen","label":{"en":"Queen","es":"Queen"},"icon":"partner","sublabel":{"en":"Most popular size","es":"El tamaño más popular"},"scores":{}},{"id":"king","label":{"en":"King","es":"King"},"icon":"family","sublabel":{"en":"Maximum space","es":"Espacio máximo"},"scores":{}},{"id":"cal_king","label":{"en":"Cal King","es":"Cal King"},"icon":"family","sublabel":{"en":"Extra length","es":"Largo extra"},"scores":{}}]},{"id":"partner_sleep","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Who's sharing the bed with you?","es":"¿Quién comparte la cama contigo?"},"helpText":{"en":"Who shares your bed shapes which features matter most.","es":"Esto determina qué características importan más"},"type":"single","options":[{"id":"solo","label":{"en":"Solo Sleeper","es":"Duermo Solo"},"icon":"solo","sublabel":{"en":"Just me","es":"Solo yo"},"scores":{}},{"id":"partner","label":{"en":"With a Partner","es":"Con Pareja"},"icon":"partner","sublabel":{"en":"Sharing the bed","es":"Compartimos la cama"},"scores":{"motionIsolation":2}},{"id":"family","label":{"en":"Family Bed","es":"Cama Familiar"},"icon":"family","sublabel":{"en":"Kids, pets, or both","es":"Niños, mascotas, o ambos"},"scores":{"durability":2,"motionIsolation":1}}]},{"id":"partner_disturbance","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Does your partner's movement wake you up?","es":"¿El movimiento de tu pareja te despierta?"},"helpText":{"en":"Motion isolation is one of the first upgrades you'll feel.","es":"El aislamiento de movimiento es una de las mayores mejoras en un colchón nuevo"},"type":"single","skipIf":{"question":"partner_sleep","answer":"solo"},"options":[{"id":"yes_often","label":{"en":"Yes, Often","es":"Sí, Seguido"},"icon":"motion","sublabel":{"en":"Every movement wakes me","es":"Cada movimiento me despierta"},"scores":{"motionIsolation":4,"hybrid":3,"memory":2}},{"id":"sometimes","label":{"en":"Sometimes","es":"A Veces"},"icon":"combo","sublabel":{"en":"Bigger movements bother me","es":"Los movimientos grandes me molestan"},"scores":{"motionIsolation":3,"hybrid":2}},{"id":"rarely","label":{"en":"Rarely","es":"Rara Vez"},"icon":"check","sublabel":{"en":"Light sleeper but mostly fine","es":"Sueño ligero pero generalmente bien"},"scores":{"motionIsolation":1}},{"id":"not_applicable","label":{"en":"Doesn't Apply","es":"No Aplica"},"icon":"solo","sublabel":{"en":"I sleep alone","es":"Duermo solo"},"scores":{}}]},{"id":"sleep_position","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"How do you usually sleep?","es":"¿Cómo duermes normalmente?"},"helpText":{"en":"Your sleep position is the biggest clue to the support you need.","es":"Piensa en cómo terminas naturalmente"},"type":"single","options":[{"id":"side","label":{"en":"Side Sleeper","es":"De Lado"},"icon":"side","sublabel":{"en":"Curled up","es":"Acurrucado"},"scores":{"plush":2,"pressureRelief":2,"soft":1}},{"id":"back","label":{"en":"Back Sleeper","es":"Boca Arriba"},"icon":"back","sublabel":{"en":"Flat on back","es":"Acostado de espalda"},"scores":{"support":2,"medium":2,"zoned":1}},{"id":"stomach","label":{"en":"Stomach Sleeper","es":"Boca Abajo"},"icon":"stomach","sublabel":{"en":"Face down","es":"Boca abajo"},"scores":{"firm":2,"support":1}},{"id":"combo","label":{"en":"Combination","es":"Combinación"},"icon":"combo","sublabel":{"en":"Move around","es":"Me muevo mucho"},"scores":{"medium":2,"responsive":2}},{"id":"no_idea","label":{"en":"Not Sure","es":"No Estoy Seguro"},"icon":"question","sublabel":{"en":"I wake up in weird positions","es":"Me despierto en posiciones raras"},"scores":{"medium":2,"responsive":2}}]},{"id":"body_type","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"What weight range should this mattress support?","es":"¿Qué rango de peso debe soportar este colchón?"},"helpText":{"en":"This helps us account for cushioning, support, and durability.","es":"Esto nos ayuda a considerar la amortiguación, el soporte y la durabilidad."},"type":"single","options":[{"id":"petite","label":{"en":"Under 130 lbs","es":"Menos de 130 lbs"},"icon":"cloud","sublabel":{"en":"Light support","es":"Soporte ligero"},"scores":{"plush":2,"soft":1}},{"id":"average","label":{"en":"130 to 200 lbs","es":"130 a 200 lbs"},"icon":"weight","sublabel":{"en":"Standard support","es":"Soporte estándar"},"scores":{"medium":2}},{"id":"athletic","label":{"en":"200 to 230 lbs","es":"200 a 230 lbs"},"icon":"support","sublabel":{"en":"Medium-firm support","es":"Soporte medio-firme"},"scores":{"support":2,"medium":1,"responsive":1}},{"id":"plus","label":{"en":"Over 230 lbs","es":"Más de 230 lbs"},"icon":"support","sublabel":{"en":"Maximum support","es":"Soporte máximo"},"scores":{"firm":2,"support":3,"hybrid":2,"durability":2}},{"id":"different","label":{"en":"Different weight ranges","es":"Rangos de peso diferentes"},"icon":"partner","sublabel":{"en":"Sleepers fall into different ranges","es":"Los durmientes están en rangos diferentes"},"scores":{"medium":2,"support":1,"motionIsolation":2},"hideIf":{"question":"partner_sleep","answer":"solo"}}],"copyVariants":[{"when":{"question":"partner_sleep","answerIn":["partner","family"]},"question":{"en":"What weight range should we match for the sleeper who needs more support?","es":"¿Para qué rango de peso debemos ajustar, según quien necesite más soporte?"},"helpText":{"en":"If you fall into different ranges, choose “Different weight ranges.”","es":"Si están en rangos diferentes, elige “Rangos de peso diferentes”."}}]},{"id":"temperature","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"How do you sleep temperature-wise?","es":"¿Cómo duermes en cuanto a temperatura?"},"helpText":{"en":"Sleeping hot or cold is an easy fix with the right materials.","es":"La regulación de temperatura es clave para un sueño profundo"},"type":"single","options":[{"id":"hot","label":{"en":"I Sleep Hot","es":"Duermo con Calor"},"icon":"flame","sublabel":{"en":"Night sweats, kick off covers","es":"Sudores nocturnos, quito las cobijas"},"scores":{"cooling":3,"hybrid":2}},{"id":"comfortable","label":{"en":"I'm Comfortable","es":"Estoy Cómodo"},"icon":"smile","sublabel":{"en":"No temperature issues","es":"Sin problemas de temperatura"},"scores":{}},{"id":"cold","label":{"en":"I Sleep Cold","es":"Duermo con Frío"},"icon":"snowflake","sublabel":{"en":"Need blankets to warm up","es":"Necesito cobijas para calentarme"},"scores":{"memory":1,"plush":1}},{"id":"opposite","label":{"en":"We're Opposite","es":"Somos Opuestos"},"icon":"hotcold","sublabel":{"en":"One hot, one cold","es":"Uno con calor, otro con frío"},"scores":{"cooling":2,"hybrid":1},"hideIf":{"question":"partner_sleep","answer":"solo"}}]},{"id":"firmness","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"What firmness level do you prefer?","es":"¿Qué nivel de firmeza prefieres?"},"helpText":{"en":"No wrong answer here, just slide to what feels best.","es":"Desliza a tu comodidad ideal"},"type":"slider","min":1,"max":10,"defaultValue":5,"labels":[{"en":"Soft — Sink right in","es":"Suave — Hundirse"},{"en":"Medium","es":"Medio"},{"en":"Firm — Solid support","es":"Firme — Soporte sólido"}]},{"id":"sleep_issues","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Any issues with your current mattress?","es":"¿Algún problema con tu colchón actual?"},"helpText":{"en":"Tap anything you've noticed. Each one points us toward a fix.","es":"Toca las que apliquen"},"type":"multiple","options":[{"id":"back_pain","label":{"en":"Back Pain","es":"Dolor de Espalda"},"icon":"spine","sublabel":{"en":"Lower or upper back","es":"Espalda baja o alta"},"scores":{"support":3,"zoned":2,"firm":1}},{"id":"hip_pain","label":{"en":"Hip or Shoulder Pain","es":"Dolor de Cadera u Hombro"},"icon":"pressure","sublabel":{"en":"Pressure points","es":"Puntos de presión"},"scores":{"pressureRelief":3,"plush":2}},{"id":"hot","label":{"en":"Sleeping Too Hot","es":"Mucho Calor al Dormir"},"icon":"flame","sublabel":{"en":"Night sweats, overheating","es":"Sudores nocturnos, sobrecalentamiento"},"scores":{"cooling":3,"hybrid":2}},{"id":"tossing","label":{"en":"Tossing &amp; Turning","es":"Dando Vueltas"},"icon":"combo","sublabel":{"en":"Can't get comfortable","es":"No encuentro comodidad"},"scores":{"comfort":2,"medium":1}},{"id":"stiff","label":{"en":"Waking Up Stiff or Sore","es":"Despertar Rígido o Adolorido"},"icon":"stiff","sublabel":{"en":"Morning aches","es":"Dolores matutinos"},"scores":{"pressureRelief":2,"comfort":2}},{"id":"sagging","label":{"en":"Mattress Sagging","es":"Colchón Hundido"},"icon":"sagging","sublabel":{"en":"Dips or indentations","es":"Hundimientos"},"scores":{"durability":2,"quality":2}},{"id":"too_soft","label":{"en":"Mattress Too Soft","es":"Colchón Muy Suave"},"icon":"couch","sublabel":{"en":"Sinking in too much","es":"Me hundo demasiado"},"scores":{"firm":3,"support":2}},{"id":"none","label":{"en":"No Major Issues","es":"Sin Problemas Grandes"},"icon":"check","sublabel":{"en":"Just time for an upgrade","es":"Solo es hora de un cambio"},"scores":{"comfort":1,"quality":1,"durable":1}}]},{"id":"health_conditions","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Anything else going on that affects your sleep?","es":"¿Algo más que afecte tu sueño?"},"helpText":{"en":"Tap any that apply. A few of these change what we'd suggest.","es":"Toca las que apliquen"},"type":"multiple","options":[{"id":"nerve_pain","label":{"en":"Nerve Pain or Tingling","es":"Dolor Nervioso u Hormigueo"},"icon":"lightning","sublabel":{"en":"Shooting pain, numbness","es":"Dolor punzante, entumecimiento"},"scores":{"support":3,"firm":2,"zoned":2}},{"id":"allergies","label":{"en":"Allergies","es":"Alergias"},"icon":"sneeze","sublabel":{"en":"Dust, sneezing, stuffy","es":"Polvo, estornudos, congestión"},"scores":{"hypoallergenic":3}},{"id":"snoring","label":{"en":"Snoring or Sleep Apnea","es":"Ronquidos o Apnea del Sueño"},"icon":"snore","sublabel":{"en":"You or your partner","es":"Tú o tu pareja"},"scores":{"adjustable":3}},{"id":"reflux","label":{"en":"Acid Reflux / Heartburn","es":"Reflujo Ácido / Acidez"},"icon":"flame","sublabel":{"en":"Burns when lying down","es":"Arde al acostarse"},"scores":{"adjustable":3}},{"id":"extra_support","label":{"en":"Need Extra Support","es":"Necesito Soporte Extra"},"icon":"weight","sublabel":{"en":"Larger build or heavier weight","es":"Complexión grande o peso mayor"},"scores":{"support":3,"firm":2,"durable":3}},{"id":"getting_older","label":{"en":"Changing Needs","es":"Necesidades Cambiantes"},"icon":"aging","sublabel":{"en":"Looking for gentler support","es":"Buscando soporte más suave"},"scores":{"support":2,"comfort":2,"pressureRelief":1}},{"id":"none","label":{"en":"None of These","es":"Ninguno de Estos"},"icon":"check","sublabel":{"en":"I'm good","es":"Estoy bien"},"scores":{}}]}]}}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Retire unsupported display claims on g6/g7/s3/g8/g9 with total component omission
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/incoming/Lacks_Store_Data.xlsx
+++ b/incoming/Lacks_Store_Data.xlsx
@@ -2289,11 +2289,7 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Hand-made plush luxury hybrid</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>1</v>
       </c>
@@ -2309,14 +2305,10 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Hand-Made|Plush|Natural Materials</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Hand-made in Texas — plush euro-top luxury</t>
-        </is>
-      </c>
+          <t>Plush</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2335,46 +2327,18 @@
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>A hand-made hybrid of natural materials with a plush euro-top — built by Restonic craftspeople to last a lifetime.</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>Hand-made plush luxury with natural materials, made regionally by Restonic.</t>
-        </is>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>Hand-made construction</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>Assembled by hand with natural materials most factory beds skip.</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>Plush euro-top feel</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>Cushioned sink-in comfort over a supportive hybrid core.</t>
-        </is>
-      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>Hecho a Mano|Suave|Materiales Naturales</t>
-        </is>
-      </c>
-      <c r="AF7" t="inlineStr">
-        <is>
-          <t>Hecho a mano en Texas — lujo suave con euro-top</t>
-        </is>
-      </c>
+          <t>Suave</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
       <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr"/>
@@ -2383,36 +2347,12 @@
       <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>Un híbrido hecho a mano con materiales naturales y euro-top suave — construido por artesanos de Restonic para durar toda la vida.</t>
-        </is>
-      </c>
-      <c r="AP7" t="inlineStr">
-        <is>
-          <t>Lujo suave hecho a mano con materiales naturales, fabricado regionalmente por Restonic.</t>
-        </is>
-      </c>
-      <c r="AQ7" t="inlineStr">
-        <is>
-          <t>Construcción a mano</t>
-        </is>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>Ensamblado a mano con materiales naturales que la mayoría de las camas de fábrica omiten.</t>
-        </is>
-      </c>
-      <c r="AS7" t="inlineStr">
-        <is>
-          <t>Sensación de euro-top suave</t>
-        </is>
-      </c>
-      <c r="AT7" t="inlineStr">
-        <is>
-          <t>Confort acolchado y envolvente sobre un núcleo híbrido de soporte.</t>
-        </is>
-      </c>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2441,11 +2381,7 @@
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Hand-made balanced luxury hybrid</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>1</v>
       </c>
@@ -2461,14 +2397,10 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Hand-Made|Medium|Natural Materials</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Hand-made balanced luxury with natural materials</t>
-        </is>
-      </c>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2487,42 +2419,18 @@
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>Hand-made with natural materials in a balanced medium tight-top — luxury that works for almost every sleeper.</t>
-        </is>
-      </c>
+      <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>True balanced medium</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>Neither plush nor firm — a safe luxury pick for couples who disagree.</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>Natural-material build</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>Hand-made with breathable natural layers built to outlast foam-only beds.</t>
-        </is>
-      </c>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>Hecho a Mano|Medio|Materiales Naturales</t>
-        </is>
-      </c>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t>Lujo equilibrado hecho a mano con materiales naturales</t>
-        </is>
-      </c>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr"/>
@@ -2531,32 +2439,12 @@
       <c r="AL8" t="inlineStr"/>
       <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr">
-        <is>
-          <t>Hecho a mano con materiales naturales en un tight-top medio equilibrado — lujo que funciona para casi todos.</t>
-        </is>
-      </c>
+      <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="inlineStr">
-        <is>
-          <t>Medio verdaderamente equilibrado</t>
-        </is>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>Ni suave ni firme — una elección de lujo segura para parejas que no se ponen de acuerdo.</t>
-        </is>
-      </c>
-      <c r="AS8" t="inlineStr">
-        <is>
-          <t>Construcción de materiales naturales</t>
-        </is>
-      </c>
-      <c r="AT8" t="inlineStr">
-        <is>
-          <t>Hecho a mano con capas naturales transpirables que duran más que las camas de pura espuma.</t>
-        </is>
-      </c>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2585,11 +2473,7 @@
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Hand-made extra-firm luxury</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>1</v>
       </c>
@@ -2605,14 +2489,10 @@
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Hand-Made|Extra Firm|Natural Materials</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Hand-made extra-firm — maximum support, luxury materials</t>
-        </is>
-      </c>
+          <t>Extra Firm</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2631,38 +2511,18 @@
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>The firmest bed in the Reserve line — hand-made hybrid support with natural materials for sleepers who want maximum lift.</t>
-        </is>
-      </c>
+      <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>True extra-firm lift</t>
-        </is>
-      </c>
+      <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>Hand-made durability</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>Natural materials and hand assembly keep the firm feel from softening early.</t>
-        </is>
-      </c>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Hecho a Mano|Extra Firme|Materiales Naturales</t>
-        </is>
-      </c>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>Extra firme hecho a mano — máximo soporte, materiales de lujo</t>
-        </is>
-      </c>
+          <t>Extra Firme</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr"/>
@@ -2671,28 +2531,12 @@
       <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>La cama más firme de la línea Reserve — soporte híbrido hecho a mano con materiales naturales para quienes quieren máxima elevación.</t>
-        </is>
-      </c>
+      <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
-      <c r="AQ9" t="inlineStr">
-        <is>
-          <t>Verdadera elevación extra firme</t>
-        </is>
-      </c>
+      <c r="AQ9" t="inlineStr"/>
       <c r="AR9" t="inlineStr"/>
-      <c r="AS9" t="inlineStr">
-        <is>
-          <t>Durabilidad hecha a mano</t>
-        </is>
-      </c>
-      <c r="AT9" t="inlineStr">
-        <is>
-          <t>Los materiales naturales y el ensamblaje a mano evitan que la firmeza se ablande antes de tiempo.</t>
-        </is>
-      </c>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2721,11 +2565,7 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Copper-infused cooling hybrid</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>1</v>
       </c>
@@ -2741,14 +2581,10 @@
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Copper-Infused|Cooling|Cushion Firm</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Copper-infused cooling with cushion-firm support</t>
-        </is>
-      </c>
+          <t>Cushion Firm</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>no</t>
@@ -2767,38 +2603,18 @@
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>Patented NatuVerex copper fabric and copper-infused memory foam — a cleaner, cooler sleep over cushion-firm hybrid support.</t>
-        </is>
-      </c>
+      <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>Copper-infused sleep surface</t>
-        </is>
-      </c>
+      <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>Cushion-firm balance</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>Supportive like a firm with a thin comfort cushion — firm without the board feel.</t>
-        </is>
-      </c>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>Infusión de Cobre|Frescura|Cushion Firm</t>
-        </is>
-      </c>
-      <c r="AF10" t="inlineStr">
-        <is>
-          <t>Frescura con infusión de cobre y soporte cushion-firm</t>
-        </is>
-      </c>
+          <t>Cushion Firm</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="inlineStr"/>
@@ -2807,28 +2623,12 @@
       <c r="AL10" t="inlineStr"/>
       <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
-      <c r="AO10" t="inlineStr">
-        <is>
-          <t>Tela de cobre patentada NatuVerex y espuma viscoelástica con cobre — un sueño más limpio y fresco sobre soporte híbrido cushion-firm.</t>
-        </is>
-      </c>
+      <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
-      <c r="AQ10" t="inlineStr">
-        <is>
-          <t>Superficie con infusión de cobre</t>
-        </is>
-      </c>
+      <c r="AQ10" t="inlineStr"/>
       <c r="AR10" t="inlineStr"/>
-      <c r="AS10" t="inlineStr">
-        <is>
-          <t>Equilibrio cushion-firm</t>
-        </is>
-      </c>
-      <c r="AT10" t="inlineStr">
-        <is>
-          <t>Soporta como un firme con un cojín delgado de confort — firme sin sentirse como tabla.</t>
-        </is>
-      </c>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3153,11 +2953,7 @@
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Plush box-top zoned hybrid</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>1</v>
       </c>
@@ -3173,14 +2969,10 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Plush Box Top|Zoned Coils|Edge Support</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Deep plush box top over zoned wrapped coils</t>
-        </is>
-      </c>
+          <t>Plush Box Top</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
           <t>yes</t>
@@ -3200,37 +2992,17 @@
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>Plush box-top softness with zoned wrapped-coil support and strong edges.</t>
-        </is>
-      </c>
-      <c r="AA13" t="inlineStr">
-        <is>
-          <t>Deep box-top plush</t>
-        </is>
-      </c>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>A pillowy sewn-on top layer with more depth than a standard plush.</t>
-        </is>
-      </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>Zoned wrapped coils</t>
-        </is>
-      </c>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>Box Top Suave|Resortes Zonificados|Soporte de Borde</t>
-        </is>
-      </c>
-      <c r="AF13" t="inlineStr">
-        <is>
-          <t>Box top suave y profundo sobre resortes envueltos zonificados</t>
-        </is>
-      </c>
+          <t>Box Top Suave</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="inlineStr"/>
@@ -3240,26 +3012,10 @@
       <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
-      <c r="AP13" t="inlineStr">
-        <is>
-          <t>Suavidad box-top con soporte de resortes envueltos zonificados y bordes fuertes.</t>
-        </is>
-      </c>
-      <c r="AQ13" t="inlineStr">
-        <is>
-          <t>Suavidad box-top profunda</t>
-        </is>
-      </c>
-      <c r="AR13" t="inlineStr">
-        <is>
-          <t>Una capa superior acolchada cosida con más profundidad que un suave estándar.</t>
-        </is>
-      </c>
-      <c r="AS13" t="inlineStr">
-        <is>
-          <t>Resortes envueltos zonificados</t>
-        </is>
-      </c>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
       <c r="AT13" t="inlineStr"/>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
feat: reduce guided quiz to nine questions
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016566LadkHHXTFxi45ECTv1
</commit_message>
<xml_diff>
--- a/incoming/Lacks_Store_Data.xlsx
+++ b/incoming/Lacks_Store_Data.xlsx
@@ -5864,7 +5864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6117,7 +6117,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>trigger.pain</t>
+          <t>sleep_issues.back_pain</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -6128,7 +6128,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>here to solve a comfort problem</t>
+          <t>test lower-back support carefully</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -6138,7 +6138,7 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
-          <t>aquí para resolver un problema de comodidad</t>
+          <t>probar con cuidado el soporte lumbar</t>
         </is>
       </c>
     </row>
@@ -6150,7 +6150,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>trigger.worn_out</t>
+          <t>sleep_issues.hip_pain</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -6161,7 +6161,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>replacing an old mattress</t>
+          <t>focus on pressure relief at hips and shoulders</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -6171,7 +6171,7 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
-          <t>reemplazando un colchón viejo</t>
+          <t>enfocarse en aliviar la presión en caderas y hombros</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>trigger.moving</t>
+          <t>sleep_issues.hot</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -6194,7 +6194,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>furnishing a new space</t>
+          <t>prioritize temperature control</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -6204,7 +6204,7 @@
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
-          <t>amueblando un espacio nuevo</t>
+          <t>priorizar el control de temperatura</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6216,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>trigger.upgrade</t>
+          <t>sleep_issues.tossing</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -6227,7 +6227,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>ready for an upgrade</t>
+          <t>notice how easy it is to settle in</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -6237,7 +6237,7 @@
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
-          <t>buscando una mejora</t>
+          <t>notar qué tan fácil es acomodarse</t>
         </is>
       </c>
     </row>
@@ -6249,7 +6249,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>trigger.browsing</t>
+          <t>sleep_issues.stiff</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -6260,7 +6260,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>exploring options today</t>
+          <t>compare alignment and morning comfort</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -6270,7 +6270,7 @@
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
-          <t>explorando opciones hoy</t>
+          <t>comparar la alineación y la comodidad al despertar</t>
         </is>
       </c>
     </row>
@@ -6282,7 +6282,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>sleep_issues.back_pain</t>
+          <t>sleep_issues.sagging</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -6293,7 +6293,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>test lower-back support carefully</t>
+          <t>check for durable, consistent support</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -6303,7 +6303,7 @@
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
-          <t>probar con cuidado el soporte lumbar</t>
+          <t>revisar que el soporte sea duradero y consistente</t>
         </is>
       </c>
     </row>
@@ -6315,7 +6315,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>sleep_issues.hip_pain</t>
+          <t>sleep_issues.too_soft</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -6326,7 +6326,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>focus on pressure relief at hips and shoulders</t>
+          <t>try firmer, more supportive feels</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -6336,7 +6336,7 @@
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
-          <t>enfocarse en aliviar la presión en caderas y hombros</t>
+          <t>probar sensaciones más firmes y con más soporte</t>
         </is>
       </c>
     </row>
@@ -6348,7 +6348,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>sleep_issues.hot</t>
+          <t>sleep_issues.none</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -6357,21 +6357,13 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>prioritize temperature control</t>
-        </is>
-      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>priorizar el control de temperatura</t>
-        </is>
-      </c>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6381,7 +6373,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>sleep_issues.tossing</t>
+          <t>sleep_position.side</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -6392,7 +6384,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>notice how easy it is to settle in</t>
+          <t>prioritize shoulder and hip cushioning</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -6402,7 +6394,7 @@
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
-          <t>notar qué tan fácil es acomodarse</t>
+          <t>priorizar el acolchado de hombros y caderas</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6406,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>sleep_issues.stiff</t>
+          <t>sleep_position.back</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -6425,7 +6417,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>compare alignment and morning comfort</t>
+          <t>look for even lumbar support</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -6435,7 +6427,7 @@
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
-          <t>comparar la alineación y la comodidad al despertar</t>
+          <t>buscar soporte lumbar uniforme</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6439,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>sleep_issues.sagging</t>
+          <t>sleep_position.stomach</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -6458,7 +6450,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>check for durable, consistent support</t>
+          <t>keep the midsection supported</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -6468,7 +6460,7 @@
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
-          <t>revisar que el soporte sea duradero y consistente</t>
+          <t>mantener la zona media con soporte</t>
         </is>
       </c>
     </row>
@@ -6480,7 +6472,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>sleep_issues.too_soft</t>
+          <t>sleep_position.combo</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -6491,7 +6483,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>try firmer, more supportive feels</t>
+          <t>notice ease of movement between positions</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -6501,7 +6493,7 @@
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr">
         <is>
-          <t>probar sensaciones más firmes y con más soporte</t>
+          <t>notar la facilidad para cambiar de posición</t>
         </is>
       </c>
     </row>
@@ -6513,7 +6505,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>sleep_issues.none</t>
+          <t>sleep_position.no_idea</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -6522,13 +6514,21 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>compare a few different feels to find a starting point</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>comparar varias sensaciones para encontrar un punto de partida</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6538,7 +6538,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>sleep_position.side</t>
+          <t>health_conditions.nerve_pain</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -6549,7 +6549,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>prioritize shoulder and hip cushioning</t>
+          <t>compare gentle, even pressure relief</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -6559,7 +6559,7 @@
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
-          <t>priorizar el acolchado de hombros y caderas</t>
+          <t>comparar un alivio de presión suave y uniforme</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6571,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>sleep_position.back</t>
+          <t>health_conditions.allergies</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -6582,7 +6582,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>look for even lumbar support</t>
+          <t>ask about washable and protective covers</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -6592,7 +6592,7 @@
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
-          <t>buscar soporte lumbar uniforme</t>
+          <t>preguntar por fundas lavables y protectoras</t>
         </is>
       </c>
     </row>
@@ -6604,7 +6604,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>sleep_position.stomach</t>
+          <t>health_conditions.snoring</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -6615,7 +6615,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>keep the midsection supported</t>
+          <t>test head-of-bed elevation on an adjustable base</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -6625,7 +6625,7 @@
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
-          <t>mantener la zona media con soporte</t>
+          <t>probar la elevación de la cabecera en una base ajustable</t>
         </is>
       </c>
     </row>
@@ -6637,7 +6637,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>sleep_position.combo</t>
+          <t>health_conditions.reflux</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -6648,7 +6648,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>notice ease of movement between positions</t>
+          <t>notice how a raised upper body feels</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -6658,7 +6658,7 @@
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr">
         <is>
-          <t>notar la facilidad para cambiar de posición</t>
+          <t>notar cómo se siente el torso elevado</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>sleep_position.no_idea</t>
+          <t>health_conditions.extra_support</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -6681,7 +6681,7 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>compare a few different feels to find a starting point</t>
+          <t>prioritize reinforced, sturdy support</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -6691,7 +6691,7 @@
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr">
         <is>
-          <t>comparar varias sensaciones para encontrar un punto de partida</t>
+          <t>priorizar un soporte reforzado y resistente</t>
         </is>
       </c>
     </row>
@@ -6703,7 +6703,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>health_conditions.nerve_pain</t>
+          <t>health_conditions.getting_older</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -6714,7 +6714,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>compare gentle, even pressure relief</t>
+          <t>compare ease of getting in and out of bed</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -6724,7 +6724,7 @@
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
-          <t>comparar un alivio de presión suave y uniforme</t>
+          <t>comparar la facilidad para acostarse y levantarse</t>
         </is>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>health_conditions.allergies</t>
+          <t>health_conditions.none</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -6745,21 +6745,13 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>ask about washable and protective covers</t>
-        </is>
-      </c>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>preguntar por fundas lavables y protectoras</t>
-        </is>
-      </c>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6769,7 +6761,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>health_conditions.snoring</t>
+          <t>temperature.hot</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -6780,7 +6772,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>test head-of-bed elevation on an adjustable base</t>
+          <t>compare cooling covers and airflow</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -6790,7 +6782,7 @@
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
-          <t>probar la elevación de la cabecera en una base ajustable</t>
+          <t>comparar fundas frescas y ventilación</t>
         </is>
       </c>
     </row>
@@ -6802,7 +6794,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>health_conditions.reflux</t>
+          <t>temperature.comfortable</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -6811,21 +6803,13 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>notice how a raised upper body feels</t>
-        </is>
-      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>notar cómo se siente el torso elevado</t>
-        </is>
-      </c>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6835,7 +6819,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>health_conditions.extra_support</t>
+          <t>temperature.cold</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -6846,7 +6830,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>prioritize reinforced, sturdy support</t>
+          <t>notice warmth and cozier surface feels</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -6856,7 +6840,7 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
-          <t>priorizar un soporte reforzado y resistente</t>
+          <t>notar calidez y superficies más acogedoras</t>
         </is>
       </c>
     </row>
@@ -6868,7 +6852,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>health_conditions.getting_older</t>
+          <t>temperature.opposite</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -6879,7 +6863,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>compare ease of getting in and out of bed</t>
+          <t>compare temperature balance for two sleepers</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -6888,155 +6872,6 @@
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr">
-        <is>
-          <t>comparar la facilidad para acostarse y levantarse</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>consultation</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>health_conditions.none</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>consultation</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>temperature.hot</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>compare cooling covers and airflow</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>comparar fundas frescas y ventilación</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>consultation</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>temperature.comfortable</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>consultation</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>temperature.cold</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>notice warmth and cozier surface feels</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>notar calidez y superficies más acogedoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>consultation</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>temperature.opposite</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>compare temperature balance for two sleepers</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr">
         <is>
           <t>comparar el equilibrio de temperatura para dos personas</t>
         </is>
@@ -7094,7 +6929,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"quiz":{"questions":[{"id":"trigger","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What can we help you with today?","es":"¿En qué te podemos ayudar hoy?"},"helpText":{"en":"This doesn't change your sleep-fit ranking. It helps your specialist focus on what matters to you.","es":"Esto no cambia el orden de tus opciones. Ayuda a tu especialista a enfocarse en lo que te importa."},"type":"single","options":[{"id":"pain","label":{"en":"Back or Body Pain","es":"Dolor de Espalda o Cuerpo"},"icon":"spine","sublabel":{"en":"Current mattress is hurting me","es":"Mi colchón actual me lastima"},"scores":{}},{"id":"worn_out","label":{"en":"Old Mattress","es":"Colchón Viejo"},"icon":"sagging","sublabel":{"en":"Time for an upgrade","es":"Es hora de un cambio"},"scores":{}},{"id":"moving","label":{"en":"Moving or New Space","es":"Mudanza o Espacio Nuevo"},"icon":"family","sublabel":{"en":"New home, new bed","es":"Casa nueva, cama nueva"},"scores":{}},{"id":"upgrade","label":{"en":"Just Upgrading","es":"Mejorando"},"icon":"cloud","sublabel":{"en":"Ready for something better","es":"Listo para algo mejor"},"scores":{}},{"id":"browsing","label":{"en":"Just Browsing","es":"Solo Explorando"},"icon":"smile","sublabel":{"en":"Getting ideas, no rush","es":"Sin prisa, juntando ideas"},"scores":{}}]},{"id":"mattress_size","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What size mattress are you looking for?","es":"¿Qué tamaño de colchón buscas?"},"helpText":{"en":"We carry your selected size into the consultation. Your sleep-fit ranking is based on your comfort and support answers.","es":"Tomamos en cuenta el tamaño que elijas en la consulta. El orden de tus opciones se basa en tus respuestas sobre comodidad y soporte."},"type":"single","options":[{"id":"twin","label":{"en":"Twin","es":"Twin"},"icon":"solo","sublabel":{"en":"Kids or tight spaces","es":"Niños o espacios pequeños"},"scores":{}},{"id":"twin_xl","label":{"en":"Twin XL","es":"Twin XL"},"icon":"solo","sublabel":{"en":"Extra length, single sleeper","es":"Largo extra, una persona"},"scores":{}},{"id":"full","label":{"en":"Full","es":"Full"},"icon":"solo","sublabel":{"en":"Solo or cozy pair","es":"Solo o pareja cómoda"},"scores":{}},{"id":"queen","label":{"en":"Queen","es":"Queen"},"icon":"partner","sublabel":{"en":"Most popular size","es":"El tamaño más popular"},"scores":{}},{"id":"king","label":{"en":"King","es":"King"},"icon":"family","sublabel":{"en":"Maximum space","es":"Espacio máximo"},"scores":{}},{"id":"cal_king","label":{"en":"Cal King","es":"Cal King"},"icon":"family","sublabel":{"en":"Extra length","es":"Largo extra"},"scores":{}}]},{"id":"partner_sleep","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Who's sharing the bed with you?","es":"¿Quién comparte la cama contigo?"},"helpText":{"en":"This shapes the questions that follow and what we suggest testing together.","es":"Esto define las preguntas que siguen y lo que sugerimos probar juntos."},"type":"single","options":[{"id":"solo","label":{"en":"Solo Sleeper","es":"Duermo Solo"},"icon":"solo","sublabel":{"en":"Just me","es":"Solo yo"},"scores":{}},{"id":"partner","label":{"en":"With a Partner","es":"Con Pareja"},"icon":"partner","sublabel":{"en":"Sharing the bed","es":"Compartimos la cama"},"scores":{"motionIsolation":2}},{"id":"family","label":{"en":"Family Bed","es":"Cama Familiar"},"icon":"family","sublabel":{"en":"Kids, pets, or both","es":"Niños, mascotas, o ambos"},"scores":{"durability":2,"motionIsolation":1}}]},{"id":"partner_disturbance","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Does your partner's movement wake you up?","es":"¿El movimiento de tu pareja te despierta?"},"helpText":{"en":"The more movement wakes you, the more it shapes your matches and what we suggest testing.","es":"Cuanto más te despierte el movimiento, más influye en tus opciones y en lo que sugerimos probar."},"type":"single","skipIf":{"question":"partner_sleep","answer":"solo"},"options":[{"id":"yes_often","label":{"en":"Yes, Often","es":"Sí, Seguido"},"icon":"motion","sublabel":{"en":"Every movement wakes me","es":"Cada movimiento me despierta"},"scores":{"motionIsolation":4,"hybrid":3,"memory":2}},{"id":"sometimes","label":{"en":"Sometimes","es":"A Veces"},"icon":"combo","sublabel":{"en":"Bigger movements bother me","es":"Los movimientos grandes me molestan"},"scores":{"motionIsolation":3,"hybrid":2}},{"id":"rarely","label":{"en":"Rarely","es":"Rara Vez"},"icon":"check","sublabel":{"en":"Light sleeper but mostly fine","es":"Sueño ligero pero generalmente bien"},"scores":{"motionIsolation":1}},{"id":"not_applicable","label":{"en":"Doesn't Apply","es":"No Aplica"},"icon":"solo","sublabel":{"en":"I sleep alone","es":"Duermo solo"},"scores":{}}]},{"id":"sleep_position","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"How do you usually sleep?","es":"¿Cómo duermes normalmente?"},"helpText":{"en":"This helps us favor pressure relief, support, or a responsive feel.","es":"Esto nos ayuda a priorizar alivio de presión, soporte o una sensación con más respuesta."},"type":"single","options":[{"id":"side","label":{"en":"Side Sleeper","es":"De Lado"},"icon":"side","sublabel":{"en":"Curled up","es":"Acurrucado"},"scores":{"plush":2,"pressureRelief":2,"soft":1}},{"id":"back","label":{"en":"Back Sleeper","es":"Boca Arriba"},"icon":"back","sublabel":{"en":"Flat on back","es":"Acostado de espalda"},"scores":{"support":2,"medium":2,"zoned":1}},{"id":"stomach","label":{"en":"Stomach Sleeper","es":"Boca Abajo"},"icon":"stomach","sublabel":{"en":"Face down","es":"Boca abajo"},"scores":{"firm":2,"support":1}},{"id":"combo","label":{"en":"Combination","es":"Combinación"},"icon":"combo","sublabel":{"en":"Move around","es":"Me muevo mucho"},"scores":{"medium":2,"responsive":2}},{"id":"no_idea","label":{"en":"Not Sure","es":"No Estoy Seguro"},"icon":"question","sublabel":{"en":"I wake up in weird positions","es":"Me despierto en posiciones raras"},"scores":{"medium":2,"responsive":2}}]},{"id":"body_type","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"What weight range should this mattress support?","es":"¿Qué rango de peso debe soportar este colchón?"},"helpText":{"en":"This helps us account for cushioning, support, and durability.","es":"Esto nos ayuda a considerar la amortiguación, el soporte y la durabilidad."},"type":"single","options":[{"id":"petite","label":{"en":"Under 130 lbs","es":"Menos de 130 lbs"},"icon":"cloud","sublabel":{"en":"Light support","es":"Soporte ligero"},"scores":{"plush":2,"soft":1}},{"id":"average","label":{"en":"130 to 200 lbs","es":"130 a 200 lbs"},"icon":"weight","sublabel":{"en":"Standard support","es":"Soporte estándar"},"scores":{"medium":2}},{"id":"athletic","label":{"en":"200 to 230 lbs","es":"200 a 230 lbs"},"icon":"support","sublabel":{"en":"Medium-firm support","es":"Soporte medio-firme"},"scores":{"support":2,"medium":1,"responsive":1}},{"id":"plus","label":{"en":"Over 230 lbs","es":"Más de 230 lbs"},"icon":"support","sublabel":{"en":"Maximum support","es":"Soporte máximo"},"scores":{"firm":2,"support":3,"hybrid":2,"durability":2}},{"id":"different","label":{"en":"Different weight ranges","es":"Rangos de peso diferentes"},"icon":"partner","sublabel":{"en":"Sleepers fall into different ranges","es":"Los durmientes están en rangos diferentes"},"scores":{"medium":2,"support":1,"motionIsolation":2},"hideIf":{"question":"partner_sleep","answer":"solo"}}],"copyVariants":[{"when":{"question":"partner_sleep","answerIn":["partner","family"]},"question":{"en":"What weight range should we match for the sleeper who needs more support?","es":"¿Para qué rango de peso debemos ajustar, según quien necesite más soporte?"},"helpText":{"en":"If you fall into different ranges, choose “Different weight ranges.”","es":"Si están en rangos diferentes, elige “Rangos de peso diferentes”."}}]},{"id":"temperature","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"How do you sleep temperature-wise?","es":"¿Cómo duermes en cuanto a temperatura?"},"helpText":{"en":"If you sleep hot, we favor cooling features in your matches.","es":"Si duermes con calor, priorizamos materiales refrescantes en tus opciones."},"type":"single","options":[{"id":"hot","label":{"en":"I Sleep Hot","es":"Duermo con Calor"},"icon":"flame","sublabel":{"en":"Night sweats, kick off covers","es":"Sudores nocturnos, quito las cobijas"},"scores":{"cooling":3,"hybrid":2}},{"id":"comfortable","label":{"en":"I'm Comfortable","es":"Estoy Cómodo"},"icon":"smile","sublabel":{"en":"No temperature issues","es":"Sin problemas de temperatura"},"scores":{}},{"id":"cold","label":{"en":"I Sleep Cold","es":"Duermo con Frío"},"icon":"snowflake","sublabel":{"en":"Need blankets to warm up","es":"Necesito cobijas para calentarme"},"scores":{"memory":1,"plush":1}},{"id":"opposite","label":{"en":"We're Opposite","es":"Somos Opuestos"},"icon":"hotcold","sublabel":{"en":"One hot, one cold","es":"Uno con calor, otro con frío"},"scores":{"cooling":2,"hybrid":1},"hideIf":{"question":"partner_sleep","answer":"solo"}}]},{"id":"firmness","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"What firmness level do you prefer?","es":"¿Qué nivel de firmeza prefieres?"},"helpText":{"en":"No wrong answer here, just slide to the feel you prefer.","es":"Desliza a tu comodidad ideal"},"type":"slider","min":1,"max":10,"defaultValue":5,"labels":[{"en":"Soft — Sink right in","es":"Suave — Hundirse"},{"en":"Medium","es":"Medio"},{"en":"Firm — Solid support","es":"Firme — Soporte sólido"}]},{"id":"sleep_issues","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Any issues with your current mattress?","es":"¿Algún problema con tu colchón actual?"},"helpText":{"en":"Tap anything you've noticed. These shape which features we favor and what we suggest testing.","es":"Toca lo que hayas notado. Esto define qué características priorizamos y qué sugerimos probar."},"type":"multiple","options":[{"id":"back_pain","label":{"en":"Back Pain","es":"Dolor de Espalda"},"icon":"spine","sublabel":{"en":"Lower or upper back","es":"Espalda baja o alta"},"scores":{"support":3,"zoned":2,"firm":1}},{"id":"hip_pain","label":{"en":"Hip or Shoulder Pain","es":"Dolor de Cadera u Hombro"},"icon":"pressure","sublabel":{"en":"Pressure points","es":"Puntos de presión"},"scores":{"pressureRelief":3,"plush":2}},{"id":"hot","label":{"en":"Sleeping Too Hot","es":"Mucho Calor al Dormir"},"icon":"flame","sublabel":{"en":"Night sweats, overheating","es":"Sudores nocturnos, sobrecalentamiento"},"scores":{"cooling":3,"hybrid":2}},{"id":"tossing","label":{"en":"Tossing &amp; Turning","es":"Dando Vueltas"},"icon":"combo","sublabel":{"en":"Can't get comfortable","es":"No encuentro comodidad"},"scores":{"comfort":2,"medium":1}},{"id":"stiff","label":{"en":"Waking Up Stiff or Sore","es":"Despertar Rígido o Adolorido"},"icon":"stiff","sublabel":{"en":"Morning aches","es":"Dolores matutinos"},"scores":{"pressureRelief":2,"comfort":2}},{"id":"sagging","label":{"en":"Mattress Sagging","es":"Colchón Hundido"},"icon":"sagging","sublabel":{"en":"Dips or indentations","es":"Hundimientos"},"scores":{"durability":2,"quality":2}},{"id":"too_soft","label":{"en":"Mattress Too Soft","es":"Colchón Muy Suave"},"icon":"couch","sublabel":{"en":"Sinking in too much","es":"Me hundo demasiado"},"scores":{"firm":3,"support":2}},{"id":"none","label":{"en":"No Major Issues","es":"Sin Problemas Grandes"},"icon":"check","sublabel":{"en":"Just time for an upgrade","es":"Solo es hora de un cambio"},"scores":{"comfort":1,"quality":1,"durable":1}}]},{"id":"health_conditions","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Anything else going on that affects your sleep?","es":"¿Algo más que afecte tu sueño?"},"helpText":{"en":"Tap any that apply. Some shape your matches; some change what we suggest trying, like an adjustable base or a mattress protector.","es":"Toca lo que aplique. Algunas influyen en tus opciones; otras cambian lo que sugerimos probar, como una base ajustable o un protector de colchón."},"type":"multiple","options":[{"id":"nerve_pain","label":{"en":"Nerve Pain or Tingling","es":"Dolor Nervioso u Hormigueo"},"icon":"lightning","sublabel":{"en":"Shooting pain, numbness","es":"Dolor punzante, entumecimiento"},"scores":{"support":3,"firm":2,"zoned":2}},{"id":"allergies","label":{"en":"Allergies","es":"Alergias"},"icon":"sneeze","sublabel":{"en":"Dust, sneezing, stuffy","es":"Polvo, estornudos, congestión"},"scores":{"hypoallergenic":3}},{"id":"snoring","label":{"en":"Snoring or Sleep Apnea","es":"Ronquidos o Apnea del Sueño"},"icon":"snore","sublabel":{"en":"You or your partner","es":"Tú o tu pareja"},"scores":{"adjustable":3}},{"id":"reflux","label":{"en":"Acid Reflux / Heartburn","es":"Reflujo Ácido / Acidez"},"icon":"flame","sublabel":{"en":"Burns when lying down","es":"Arde al acostarse"},"scores":{"adjustable":3}},{"id":"extra_support","label":{"en":"Need Extra Support","es":"Necesito Soporte Extra"},"icon":"weight","sublabel":{"en":"Larger build or heavier weight","es":"Complexión grande o peso mayor"},"scores":{"support":3,"firm":2,"durable":3}},{"id":"getting_older","label":{"en":"Changing Needs","es":"Necesidades Cambiantes"},"icon":"aging","sublabel":{"en":"Looking for gentler support","es":"Buscando soporte más suave"},"scores":{"support":2,"comfort":2,"pressureRelief":1}},{"id":"none","label":{"en":"None of These","es":"Ninguno de Estos"},"icon":"check","sublabel":{"en":"I'm good","es":"Estoy bien"},"scores":{}}]}]}}</t>
+          <t>{"quiz":{"questions":[{"id":"mattress_size","category":{"en":"Getting Started","es":"Para Empezar"},"question":{"en":"What size mattress are you looking for?","es":"¿Qué tamaño de colchón buscas?"},"helpText":{"en":"We carry your selected size into the consultation. Your sleep-fit ranking is based on your comfort and support answers.","es":"Tomamos en cuenta el tamaño que elijas en la consulta. El orden de tus opciones se basa en tus respuestas sobre comodidad y soporte."},"type":"single","options":[{"id":"twin","label":{"en":"Twin","es":"Twin"},"icon":"solo","sublabel":{"en":"Kids or tight spaces","es":"Niños o espacios pequeños"},"scores":{}},{"id":"twin_xl","label":{"en":"Twin XL","es":"Twin XL"},"icon":"solo","sublabel":{"en":"Extra length, single sleeper","es":"Largo extra, una persona"},"scores":{}},{"id":"full","label":{"en":"Full","es":"Full"},"icon":"solo","sublabel":{"en":"Solo or cozy pair","es":"Solo o pareja cómoda"},"scores":{}},{"id":"queen","label":{"en":"Queen","es":"Queen"},"icon":"partner","sublabel":{"en":"Most popular size","es":"El tamaño más popular"},"scores":{}},{"id":"king","label":{"en":"King","es":"King"},"icon":"family","sublabel":{"en":"Maximum space","es":"Espacio máximo"},"scores":{}},{"id":"cal_king","label":{"en":"Cal King","es":"Cal King"},"icon":"family","sublabel":{"en":"Extra length","es":"Largo extra"},"scores":{}}]},{"id":"partner_sleep","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Who's sharing the bed with you?","es":"¿Quién comparte la cama contigo?"},"helpText":{"en":"This shapes the questions that follow and what we suggest testing together.","es":"Esto define las preguntas que siguen y lo que sugerimos probar juntos."},"type":"single","options":[{"id":"solo","label":{"en":"Solo Sleeper","es":"Duermo Solo"},"icon":"solo","sublabel":{"en":"Just me","es":"Solo yo"},"scores":{}},{"id":"partner","label":{"en":"With a Partner","es":"Con Pareja"},"icon":"partner","sublabel":{"en":"Sharing the bed","es":"Compartimos la cama"},"scores":{"motionIsolation":2}},{"id":"family","label":{"en":"Family Bed","es":"Cama Familiar"},"icon":"family","sublabel":{"en":"Kids, pets, or both","es":"Niños, mascotas, o ambos"},"scores":{"durability":2,"motionIsolation":1}}]},{"id":"partner_disturbance","category":{"en":"Who's With You","es":"Quién Está Contigo"},"question":{"en":"Does your partner's movement wake you up?","es":"¿El movimiento de tu pareja te despierta?"},"helpText":{"en":"The more movement wakes you, the more it shapes your matches and what we suggest testing.","es":"Cuanto más te despierte el movimiento, más influye en tus opciones y en lo que sugerimos probar."},"type":"single","skipIf":{"question":"partner_sleep","answer":"solo"},"options":[{"id":"yes_often","label":{"en":"Yes, Often","es":"Sí, Seguido"},"icon":"motion","sublabel":{"en":"Every movement wakes me","es":"Cada movimiento me despierta"},"scores":{"motionIsolation":4,"hybrid":3,"memory":2}},{"id":"sometimes","label":{"en":"Sometimes","es":"A Veces"},"icon":"combo","sublabel":{"en":"Bigger movements bother me","es":"Los movimientos grandes me molestan"},"scores":{"motionIsolation":3,"hybrid":2}},{"id":"rarely","label":{"en":"Rarely","es":"Rara Vez"},"icon":"check","sublabel":{"en":"Light sleeper but mostly fine","es":"Sueño ligero pero generalmente bien"},"scores":{"motionIsolation":1}},{"id":"not_applicable","label":{"en":"Doesn't Apply","es":"No Aplica"},"icon":"solo","sublabel":{"en":"I sleep alone","es":"Duermo solo"},"scores":{}}]},{"id":"sleep_position","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"How do you usually sleep?","es":"¿Cómo duermes normalmente?"},"helpText":{"en":"This helps us favor pressure relief, support, or a responsive feel.","es":"Esto nos ayuda a priorizar alivio de presión, soporte o una sensación con más respuesta."},"type":"single","options":[{"id":"side","label":{"en":"Side Sleeper","es":"De Lado"},"icon":"side","sublabel":{"en":"Curled up","es":"Acurrucado"},"scores":{"plush":2,"pressureRelief":2,"soft":1}},{"id":"back","label":{"en":"Back Sleeper","es":"Boca Arriba"},"icon":"back","sublabel":{"en":"Flat on back","es":"Acostado de espalda"},"scores":{"support":2,"medium":2,"zoned":1}},{"id":"stomach","label":{"en":"Stomach Sleeper","es":"Boca Abajo"},"icon":"stomach","sublabel":{"en":"Face down","es":"Boca abajo"},"scores":{"firm":2,"support":1}},{"id":"combo","label":{"en":"Combination","es":"Combinación"},"icon":"combo","sublabel":{"en":"Move around","es":"Me muevo mucho"},"scores":{"medium":2,"responsive":2}},{"id":"no_idea","label":{"en":"Not Sure","es":"No Estoy Seguro"},"icon":"question","sublabel":{"en":"I wake up in weird positions","es":"Me despierto en posiciones raras"},"scores":{"medium":2,"responsive":2}}]},{"id":"body_type","category":{"en":"About You","es":"Sobre Ti"},"question":{"en":"What weight range should this mattress support?","es":"¿Qué rango de peso debe soportar este colchón?"},"helpText":{"en":"This helps us account for cushioning, support, and durability.","es":"Esto nos ayuda a considerar la amortiguación, el soporte y la durabilidad."},"type":"single","options":[{"id":"petite","label":{"en":"Under 130 lbs","es":"Menos de 130 lbs"},"icon":"cloud","sublabel":{"en":"Light support","es":"Soporte ligero"},"scores":{"plush":2,"soft":1}},{"id":"average","label":{"en":"130 to 200 lbs","es":"130 a 200 lbs"},"icon":"weight","sublabel":{"en":"Standard support","es":"Soporte estándar"},"scores":{"medium":2}},{"id":"athletic","label":{"en":"200 to 230 lbs","es":"200 a 230 lbs"},"icon":"support","sublabel":{"en":"Medium-firm support","es":"Soporte medio-firme"},"scores":{"support":2,"medium":1,"responsive":1}},{"id":"plus","label":{"en":"Over 230 lbs","es":"Más de 230 lbs"},"icon":"support","sublabel":{"en":"Maximum support","es":"Soporte máximo"},"scores":{"firm":2,"support":3,"hybrid":2,"durability":2}},{"id":"different","label":{"en":"Different weight ranges","es":"Rangos de peso diferentes"},"icon":"partner","sublabel":{"en":"Sleepers fall into different ranges","es":"Los durmientes están en rangos diferentes"},"scores":{"medium":2,"support":1,"motionIsolation":2},"hideIf":{"question":"partner_sleep","answer":"solo"}}],"copyVariants":[{"when":{"question":"partner_sleep","answerIn":["partner","family"]},"question":{"en":"What weight range should we match for the sleeper who needs more support?","es":"¿Para qué rango de peso debemos ajustar, según quien necesite más soporte?"},"helpText":{"en":"If you fall into different ranges, choose “Different weight ranges.”","es":"Si están en rangos diferentes, elige “Rangos de peso diferentes”."}}]},{"id":"temperature","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"How do you sleep temperature-wise?","es":"¿Cómo duermes en cuanto a temperatura?"},"helpText":{"en":"If you sleep hot, we favor cooling features in your matches.","es":"Si duermes con calor, priorizamos materiales refrescantes en tus opciones."},"type":"single","options":[{"id":"hot","label":{"en":"I Sleep Hot","es":"Duermo con Calor"},"icon":"flame","sublabel":{"en":"Night sweats, kick off covers","es":"Sudores nocturnos, quito las cobijas"},"scores":{"cooling":3,"hybrid":2}},{"id":"comfortable","label":{"en":"I'm Comfortable","es":"Estoy Cómodo"},"icon":"smile","sublabel":{"en":"No temperature issues","es":"Sin problemas de temperatura"},"scores":{}},{"id":"cold","label":{"en":"I Sleep Cold","es":"Duermo con Frío"},"icon":"snowflake","sublabel":{"en":"Need blankets to warm up","es":"Necesito cobijas para calentarme"},"scores":{"memory":1,"plush":1}},{"id":"opposite","label":{"en":"We're Opposite","es":"Somos Opuestos"},"icon":"hotcold","sublabel":{"en":"One hot, one cold","es":"Uno con calor, otro con frío"},"scores":{"cooling":2,"hybrid":1},"hideIf":{"question":"partner_sleep","answer":"solo"}}]},{"id":"firmness","category":{"en":"What You Like","es":"Lo Que Te Gusta"},"question":{"en":"What firmness level do you prefer?","es":"¿Qué nivel de firmeza prefieres?"},"helpText":{"en":"No wrong answer here, just slide to the feel you prefer.","es":"Desliza a tu comodidad ideal"},"type":"slider","min":1,"max":10,"defaultValue":5,"labels":[{"en":"Soft — Sink right in","es":"Suave — Hundirse"},{"en":"Medium","es":"Medio"},{"en":"Firm — Solid support","es":"Firme — Soporte sólido"}]},{"id":"sleep_issues","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Any issues with your current mattress?","es":"¿Algún problema con tu colchón actual?"},"helpText":{"en":"Tap anything you've noticed. These shape which features we favor and what we suggest testing.","es":"Toca lo que hayas notado. Esto define qué características priorizamos y qué sugerimos probar."},"type":"multiple","options":[{"id":"back_pain","label":{"en":"Back Pain","es":"Dolor de Espalda"},"icon":"spine","sublabel":{"en":"Lower or upper back","es":"Espalda baja o alta"},"scores":{"support":3,"zoned":2,"firm":1}},{"id":"hip_pain","label":{"en":"Hip or Shoulder Pain","es":"Dolor de Cadera u Hombro"},"icon":"pressure","sublabel":{"en":"Pressure points","es":"Puntos de presión"},"scores":{"pressureRelief":3,"plush":2}},{"id":"hot","label":{"en":"Sleeping Too Hot","es":"Mucho Calor al Dormir"},"icon":"flame","sublabel":{"en":"Night sweats, overheating","es":"Sudores nocturnos, sobrecalentamiento"},"scores":{"cooling":3,"hybrid":2}},{"id":"tossing","label":{"en":"Tossing &amp; Turning","es":"Dando Vueltas"},"icon":"combo","sublabel":{"en":"Can't get comfortable","es":"No encuentro comodidad"},"scores":{"comfort":2,"medium":1}},{"id":"stiff","label":{"en":"Waking Up Stiff or Sore","es":"Despertar Rígido o Adolorido"},"icon":"stiff","sublabel":{"en":"Morning aches","es":"Dolores matutinos"},"scores":{"pressureRelief":2,"comfort":2}},{"id":"sagging","label":{"en":"Mattress Sagging","es":"Colchón Hundido"},"icon":"sagging","sublabel":{"en":"Dips or indentations","es":"Hundimientos"},"scores":{"durability":2,"quality":2}},{"id":"too_soft","label":{"en":"Mattress Too Soft","es":"Colchón Muy Suave"},"icon":"couch","sublabel":{"en":"Sinking in too much","es":"Me hundo demasiado"},"scores":{"firm":3,"support":2}},{"id":"none","label":{"en":"No Major Issues","es":"Sin Problemas Grandes"},"icon":"check","sublabel":{"en":"Just time for an upgrade","es":"Solo es hora de un cambio"},"scores":{"comfort":1,"quality":1,"durable":1}}]},{"id":"health_conditions","category":{"en":"What You're Solving","es":"Lo Que Buscas Resolver"},"question":{"en":"Anything else going on that affects your sleep?","es":"¿Algo más que afecte tu sueño?"},"helpText":{"en":"Tap any that apply. Some shape your matches; some change what we suggest trying, like an adjustable base or a mattress protector.","es":"Toca lo que aplique. Algunas influyen en tus opciones; otras cambian lo que sugerimos probar, como una base ajustable o un protector de colchón."},"type":"multiple","options":[{"id":"nerve_pain","label":{"en":"Nerve Pain or Tingling","es":"Dolor Nervioso u Hormigueo"},"icon":"lightning","sublabel":{"en":"Shooting pain, numbness","es":"Dolor punzante, entumecimiento"},"scores":{"support":3,"firm":2,"zoned":2}},{"id":"allergies","label":{"en":"Allergies","es":"Alergias"},"icon":"sneeze","sublabel":{"en":"Dust, sneezing, stuffy","es":"Polvo, estornudos, congestión"},"scores":{"hypoallergenic":3}},{"id":"snoring","label":{"en":"Snoring or Sleep Apnea","es":"Ronquidos o Apnea del Sueño"},"icon":"snore","sublabel":{"en":"You or your partner","es":"Tú o tu pareja"},"scores":{"adjustable":3}},{"id":"reflux","label":{"en":"Acid Reflux / Heartburn","es":"Reflujo Ácido / Acidez"},"icon":"flame","sublabel":{"en":"Burns when lying down","es":"Arde al acostarse"},"scores":{"adjustable":3}},{"id":"extra_support","label":{"en":"Need Extra Support","es":"Necesito Soporte Extra"},"icon":"weight","sublabel":{"en":"Larger build or heavier weight","es":"Complexión grande o peso mayor"},"scores":{"support":3,"firm":2,"durable":3}},{"id":"getting_older","label":{"en":"Changing Needs","es":"Necesidades Cambiantes"},"icon":"aging","sublabel":{"en":"Looking for gentler support","es":"Buscando soporte más suave"},"scores":{"support":2,"comfort":2,"pressureRelief":1}},{"id":"none","label":{"en":"None of These","es":"Ninguno de Estos"},"icon":"check","sublabel":{"en":"I'm good","es":"Estoy bien"},"scores":{}}]}]}}</t>
         </is>
       </c>
     </row>

</xml_diff>